<commit_message>
CV filter panel: resizable sidebar, sub-grouped Funding Agency, UX polish
- CP Divider: draggable sidebar resize handle (120–520px, amber colour)
- CP Scroll: amber hover/active states on filter scrollbar
- Category labels in canvas label column now use their category colour
- .js file drag-and-drop support (parses window.__TIMELINE_DATA__)
- Funding Agency accordion sub-groups: Tri-council, Concordia, Other
  - Tri-council: SSHRC, NSERC, CFREF, CFI, New Frontiers in Research Fund
  - Concordia: Fine Arts, Fine Arts-Engineering, Office of Research,
    Jarislowsky Institute, Concordia University
  - Both Fonds variants normalised to "Fonds de recherche du Québec"
  - Concordia agency names drop redundant "Concordia" prefix / "Faculty"
  - Sub-groups are themselves collapsible accordions
- Filter section order: Institution → Funding Agency → Categories → Role

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/cv-data/cv.xlsx
+++ b/data/cv-data/cv.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H286"/>
+  <dimension ref="A1:I286"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -424,6 +424,7 @@
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="36" customWidth="1" min="7" max="7"/>
     <col width="51" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -467,6 +468,11 @@
           <t>program</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>funding_group</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -501,6 +507,7 @@
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -535,6 +542,7 @@
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -569,6 +577,7 @@
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -603,6 +612,7 @@
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -637,6 +647,7 @@
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -671,6 +682,7 @@
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -705,6 +717,7 @@
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -739,6 +752,7 @@
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -773,6 +787,7 @@
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -807,6 +822,7 @@
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -841,6 +857,7 @@
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -875,6 +892,7 @@
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -909,6 +927,7 @@
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -943,6 +962,7 @@
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -969,6 +989,7 @@
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -999,6 +1020,7 @@
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1025,6 +1047,7 @@
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1051,6 +1074,7 @@
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1077,6 +1101,7 @@
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1103,6 +1128,7 @@
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1129,6 +1155,7 @@
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1155,6 +1182,7 @@
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1181,6 +1209,7 @@
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1207,6 +1236,7 @@
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1233,6 +1263,7 @@
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1259,6 +1290,7 @@
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1289,6 +1321,7 @@
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1315,6 +1348,7 @@
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1341,6 +1375,7 @@
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1371,6 +1406,7 @@
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1401,6 +1437,7 @@
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1427,6 +1464,7 @@
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1453,6 +1491,7 @@
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1479,6 +1518,7 @@
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1505,6 +1545,7 @@
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1531,6 +1572,7 @@
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1557,6 +1599,7 @@
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1587,6 +1630,7 @@
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1613,6 +1657,7 @@
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1639,6 +1684,7 @@
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1673,6 +1719,7 @@
         </is>
       </c>
       <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1707,6 +1754,7 @@
         </is>
       </c>
       <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1741,6 +1789,7 @@
         </is>
       </c>
       <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1771,6 +1820,7 @@
       </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1801,6 +1851,7 @@
       </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1831,6 +1882,7 @@
       </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1861,6 +1913,7 @@
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1891,6 +1944,7 @@
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1921,6 +1975,7 @@
       </c>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1951,6 +2006,7 @@
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1981,6 +2037,7 @@
       </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2011,6 +2068,7 @@
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2041,6 +2099,7 @@
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2071,6 +2130,7 @@
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2101,6 +2161,7 @@
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2131,6 +2192,7 @@
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2161,6 +2223,7 @@
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2191,6 +2254,7 @@
       </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2221,6 +2285,7 @@
       </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2251,6 +2316,7 @@
       </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2281,6 +2347,7 @@
       </c>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2311,6 +2378,7 @@
       </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2341,6 +2409,7 @@
       </c>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2371,6 +2440,7 @@
       </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2401,6 +2471,7 @@
       </c>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2431,6 +2502,7 @@
       </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2461,6 +2533,7 @@
       </c>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2491,6 +2564,7 @@
       </c>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2521,6 +2595,7 @@
       </c>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2551,6 +2626,7 @@
       </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2581,6 +2657,7 @@
       </c>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2611,6 +2688,7 @@
       </c>
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2641,6 +2719,7 @@
       </c>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2671,6 +2750,7 @@
       </c>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2701,6 +2781,7 @@
       </c>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2731,6 +2812,7 @@
       </c>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2761,6 +2843,7 @@
       </c>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2791,6 +2874,7 @@
       </c>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2821,6 +2905,7 @@
       </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2851,6 +2936,7 @@
       </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2881,6 +2967,7 @@
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2911,6 +2998,7 @@
       </c>
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2941,6 +3029,7 @@
       </c>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2971,6 +3060,7 @@
       </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr"/>
+      <c r="I85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3001,6 +3091,7 @@
       </c>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr"/>
+      <c r="I86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3031,6 +3122,7 @@
       </c>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr"/>
+      <c r="I87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3061,6 +3153,7 @@
       </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr"/>
+      <c r="I88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3091,6 +3184,7 @@
       </c>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr"/>
+      <c r="I89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3121,6 +3215,7 @@
       </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3151,6 +3246,7 @@
       </c>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3181,6 +3277,7 @@
       </c>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3211,6 +3308,7 @@
       </c>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3241,6 +3339,7 @@
       </c>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3271,6 +3370,7 @@
       </c>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3301,6 +3401,7 @@
       </c>
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3331,6 +3432,7 @@
       </c>
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3361,6 +3463,7 @@
       </c>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr"/>
+      <c r="I98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3391,6 +3494,7 @@
       </c>
       <c r="G99" t="inlineStr"/>
       <c r="H99" t="inlineStr"/>
+      <c r="I99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3421,6 +3525,7 @@
       </c>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr"/>
+      <c r="I100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3451,6 +3556,7 @@
       </c>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="inlineStr"/>
+      <c r="I101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -3481,6 +3587,7 @@
       </c>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="inlineStr"/>
+      <c r="I102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -3511,6 +3618,7 @@
       </c>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr"/>
+      <c r="I103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -3541,6 +3649,7 @@
       </c>
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="inlineStr"/>
+      <c r="I104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -3571,6 +3680,7 @@
       </c>
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="inlineStr"/>
+      <c r="I105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -3601,6 +3711,7 @@
       </c>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="inlineStr"/>
+      <c r="I106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -3631,6 +3742,7 @@
       </c>
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr"/>
+      <c r="I107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -3661,6 +3773,7 @@
       </c>
       <c r="G108" t="inlineStr"/>
       <c r="H108" t="inlineStr"/>
+      <c r="I108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -3691,6 +3804,7 @@
       </c>
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr"/>
+      <c r="I109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -3721,6 +3835,7 @@
       </c>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr"/>
+      <c r="I110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -3751,6 +3866,7 @@
       </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr"/>
+      <c r="I111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -3781,6 +3897,7 @@
       </c>
       <c r="G112" t="inlineStr"/>
       <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -3811,6 +3928,7 @@
       </c>
       <c r="G113" t="inlineStr"/>
       <c r="H113" t="inlineStr"/>
+      <c r="I113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -3841,6 +3959,7 @@
       </c>
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="inlineStr"/>
+      <c r="I114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -3871,6 +3990,7 @@
       </c>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr"/>
+      <c r="I115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -3901,6 +4021,7 @@
       </c>
       <c r="G116" t="inlineStr"/>
       <c r="H116" t="inlineStr"/>
+      <c r="I116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -3931,6 +4052,7 @@
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr"/>
+      <c r="I117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -3961,6 +4083,7 @@
       </c>
       <c r="G118" t="inlineStr"/>
       <c r="H118" t="inlineStr"/>
+      <c r="I118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -3991,6 +4114,7 @@
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="inlineStr"/>
+      <c r="I119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -4021,6 +4145,7 @@
       </c>
       <c r="G120" t="inlineStr"/>
       <c r="H120" t="inlineStr"/>
+      <c r="I120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -4051,6 +4176,7 @@
       </c>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr"/>
+      <c r="I121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -4081,6 +4207,7 @@
       </c>
       <c r="G122" t="inlineStr"/>
       <c r="H122" t="inlineStr"/>
+      <c r="I122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -4111,6 +4238,7 @@
       </c>
       <c r="G123" t="inlineStr"/>
       <c r="H123" t="inlineStr"/>
+      <c r="I123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -4141,6 +4269,7 @@
       </c>
       <c r="G124" t="inlineStr"/>
       <c r="H124" t="inlineStr"/>
+      <c r="I124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -4171,6 +4300,7 @@
       </c>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="inlineStr"/>
+      <c r="I125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -4201,6 +4331,7 @@
       </c>
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="inlineStr"/>
+      <c r="I126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -4231,6 +4362,7 @@
       </c>
       <c r="G127" t="inlineStr"/>
       <c r="H127" t="inlineStr"/>
+      <c r="I127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -4261,6 +4393,7 @@
       </c>
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="inlineStr"/>
+      <c r="I128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -4291,6 +4424,7 @@
       </c>
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="inlineStr"/>
+      <c r="I129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -4321,6 +4455,7 @@
       </c>
       <c r="G130" t="inlineStr"/>
       <c r="H130" t="inlineStr"/>
+      <c r="I130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -4351,6 +4486,7 @@
       </c>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="inlineStr"/>
+      <c r="I131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -4381,6 +4517,7 @@
       </c>
       <c r="G132" t="inlineStr"/>
       <c r="H132" t="inlineStr"/>
+      <c r="I132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -4411,6 +4548,7 @@
       </c>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="inlineStr"/>
+      <c r="I133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -4441,6 +4579,7 @@
       </c>
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="inlineStr"/>
+      <c r="I134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -4471,6 +4610,7 @@
       </c>
       <c r="G135" t="inlineStr"/>
       <c r="H135" t="inlineStr"/>
+      <c r="I135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -4501,6 +4641,7 @@
       </c>
       <c r="G136" t="inlineStr"/>
       <c r="H136" t="inlineStr"/>
+      <c r="I136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -4531,6 +4672,7 @@
       </c>
       <c r="G137" t="inlineStr"/>
       <c r="H137" t="inlineStr"/>
+      <c r="I137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -4561,6 +4703,7 @@
       </c>
       <c r="G138" t="inlineStr"/>
       <c r="H138" t="inlineStr"/>
+      <c r="I138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -4591,6 +4734,7 @@
       </c>
       <c r="G139" t="inlineStr"/>
       <c r="H139" t="inlineStr"/>
+      <c r="I139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -4621,6 +4765,7 @@
       </c>
       <c r="G140" t="inlineStr"/>
       <c r="H140" t="inlineStr"/>
+      <c r="I140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -4659,6 +4804,11 @@
           <t>Social Sciences and Humanities Research Council</t>
         </is>
       </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>Tri-council</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -4697,6 +4847,11 @@
           <t>Social Sciences and Humanities Research Council</t>
         </is>
       </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>Tri-council</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -4735,6 +4890,7 @@
           <t>Schmidt Family Foundation</t>
         </is>
       </c>
+      <c r="I143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -4773,6 +4929,11 @@
           <t>New Frontiers in Research Fund</t>
         </is>
       </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>Tri-council</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -4811,6 +4972,7 @@
           <t>The MacArthur Foundation</t>
         </is>
       </c>
+      <c r="I145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -4849,6 +5011,11 @@
           <t>Social Sciences and Humanities Research Council</t>
         </is>
       </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>Tri-council</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -4887,6 +5054,11 @@
           <t>Canada Foundation for Innovation</t>
         </is>
       </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>Tri-council</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -4925,6 +5097,7 @@
           <t>Montalvo Arts Center</t>
         </is>
       </c>
+      <c r="I148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -4963,6 +5136,7 @@
           <t>Schmidt Family Foundation</t>
         </is>
       </c>
+      <c r="I149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -5001,6 +5175,11 @@
           <t>Social Sciences and Humanities Research Council</t>
         </is>
       </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>Tri-council</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -5039,6 +5218,7 @@
           <t>Fonds de recherche du Québec</t>
         </is>
       </c>
+      <c r="I151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -5077,6 +5257,7 @@
           <t>Hewitt Foundation</t>
         </is>
       </c>
+      <c r="I152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -5115,6 +5296,7 @@
           <t>Indigenous Screen Office</t>
         </is>
       </c>
+      <c r="I153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -5153,6 +5335,7 @@
           <t>Canada Council for the Arts</t>
         </is>
       </c>
+      <c r="I154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -5191,6 +5374,11 @@
           <t>Social Sciences and Humanities Research Council</t>
         </is>
       </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>Tri-council</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -5225,6 +5413,7 @@
       </c>
       <c r="G156" t="inlineStr"/>
       <c r="H156" t="inlineStr"/>
+      <c r="I156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -5263,6 +5452,7 @@
           <t>Kanaeokana Network</t>
         </is>
       </c>
+      <c r="I157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -5301,6 +5491,7 @@
           <t>Kanaeokana Network</t>
         </is>
       </c>
+      <c r="I158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -5339,6 +5530,7 @@
           <t>Canada Council for the Arts</t>
         </is>
       </c>
+      <c r="I159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -5377,6 +5569,11 @@
           <t>Social Sciences and Humanities Research Council</t>
         </is>
       </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>Tri-council</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -5415,6 +5612,7 @@
           <t>Pierre Elliott Trudeau Foundation</t>
         </is>
       </c>
+      <c r="I161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -5453,6 +5651,11 @@
           <t>Social Sciences and Humanities Research Council</t>
         </is>
       </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>Tri-council</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -5491,6 +5694,7 @@
           <t>Canada Council for the Arts</t>
         </is>
       </c>
+      <c r="I163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -5526,9 +5730,10 @@
       <c r="G164" t="inlineStr"/>
       <c r="H164" t="inlineStr">
         <is>
-          <t>Fonds québécois de la recherche</t>
-        </is>
-      </c>
+          <t>Fonds de recherche du Québec</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -5567,6 +5772,7 @@
           <t>J. W. McConnell Family Foundation</t>
         </is>
       </c>
+      <c r="I165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -5605,6 +5811,7 @@
           <t>Canada Council for the Arts</t>
         </is>
       </c>
+      <c r="I166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -5643,6 +5850,11 @@
           <t>Social Sciences and Humanities Research Council</t>
         </is>
       </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>Tri-council</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -5681,6 +5893,7 @@
           <t>Canada Council for the Arts</t>
         </is>
       </c>
+      <c r="I168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -5719,6 +5932,7 @@
           <t>Canada Council for the Arts</t>
         </is>
       </c>
+      <c r="I169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -5754,9 +5968,10 @@
       <c r="G170" t="inlineStr"/>
       <c r="H170" t="inlineStr">
         <is>
-          <t>Fonds québécois de la recherche</t>
-        </is>
-      </c>
+          <t>Fonds de recherche du Québec</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -5792,9 +6007,10 @@
       <c r="G171" t="inlineStr"/>
       <c r="H171" t="inlineStr">
         <is>
-          <t>Fonds québécois de la recherche</t>
-        </is>
-      </c>
+          <t>Fonds de recherche du Québec</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -5833,6 +6049,11 @@
           <t>Social Sciences and Humanities Research Council</t>
         </is>
       </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>Tri-council</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -5871,6 +6092,11 @@
           <t>Social Sciences and Humanities Research Council</t>
         </is>
       </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>Tri-council</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -5909,6 +6135,7 @@
           <t>Hexagram Institute</t>
         </is>
       </c>
+      <c r="I174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -5944,9 +6171,10 @@
       <c r="G175" t="inlineStr"/>
       <c r="H175" t="inlineStr">
         <is>
-          <t>Fonds québécois de la recherche</t>
-        </is>
-      </c>
+          <t>Fonds de recherche du Québec</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -5985,6 +6213,7 @@
           <t>Hexagram Institute</t>
         </is>
       </c>
+      <c r="I176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -6023,6 +6252,7 @@
           <t>Arts Council of England</t>
         </is>
       </c>
+      <c r="I177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -6061,6 +6291,11 @@
           <t>Canada First Research Excellence Fund</t>
         </is>
       </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>Tri-council</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -6099,6 +6334,11 @@
           <t>Natural Sciences and Engineering Research Council</t>
         </is>
       </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>Tri-council</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -6137,6 +6377,11 @@
           <t>Social Sciences and Humanities Research Council</t>
         </is>
       </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>Tri-council</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -6175,6 +6420,11 @@
           <t>New Frontiers in Research Fund</t>
         </is>
       </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>Tri-council</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -6213,6 +6463,7 @@
           <t>Fonds de recherche du Québec</t>
         </is>
       </c>
+      <c r="I182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -6251,6 +6502,11 @@
           <t>Social Sciences and Humanities Research Council</t>
         </is>
       </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>Tri-council</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -6289,6 +6545,11 @@
           <t>Social Sciences and Humanities Research Council</t>
         </is>
       </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>Tri-council</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -6327,6 +6588,11 @@
           <t>Social Sciences and Humanities Research Council</t>
         </is>
       </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>Tri-council</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -6365,6 +6631,11 @@
           <t>Social Sciences and Humanities Research Council</t>
         </is>
       </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>Tri-council</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -6400,9 +6671,10 @@
       <c r="G187" t="inlineStr"/>
       <c r="H187" t="inlineStr">
         <is>
-          <t>Fonds québécois de la recherche</t>
-        </is>
-      </c>
+          <t>Fonds de recherche du Québec</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -6437,6 +6709,7 @@
       </c>
       <c r="G188" t="inlineStr"/>
       <c r="H188" t="inlineStr"/>
+      <c r="I188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -6471,6 +6744,7 @@
       </c>
       <c r="G189" t="inlineStr"/>
       <c r="H189" t="inlineStr"/>
+      <c r="I189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -6505,6 +6779,7 @@
       </c>
       <c r="G190" t="inlineStr"/>
       <c r="H190" t="inlineStr"/>
+      <c r="I190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -6539,6 +6814,7 @@
       </c>
       <c r="G191" t="inlineStr"/>
       <c r="H191" t="inlineStr"/>
+      <c r="I191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -6574,9 +6850,10 @@
       <c r="G192" t="inlineStr"/>
       <c r="H192" t="inlineStr">
         <is>
-          <t>Fonds québécois de la recherche</t>
-        </is>
-      </c>
+          <t>Fonds de recherche du Québec</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -6615,6 +6892,7 @@
           <t>Heritage Canada</t>
         </is>
       </c>
+      <c r="I193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -6650,9 +6928,10 @@
       <c r="G194" t="inlineStr"/>
       <c r="H194" t="inlineStr">
         <is>
-          <t>Fonds québécois de la recherche</t>
-        </is>
-      </c>
+          <t>Fonds de recherche du Québec</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -6691,6 +6970,7 @@
           <t>Heritage Canada</t>
         </is>
       </c>
+      <c r="I195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -6729,6 +7009,11 @@
           <t>Concordia University</t>
         </is>
       </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>Concordia</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -6767,6 +7052,11 @@
           <t>Concordia University</t>
         </is>
       </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>Concordia</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -6805,6 +7095,11 @@
           <t>Jarislowsky Institute</t>
         </is>
       </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>Concordia</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -6843,6 +7138,11 @@
           <t>Concordia University</t>
         </is>
       </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>Concordia</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -6881,6 +7181,11 @@
           <t>Concordia University</t>
         </is>
       </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>Concordia</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -6919,6 +7224,11 @@
           <t>Concordia University</t>
         </is>
       </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>Concordia</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -6954,7 +7264,12 @@
       <c r="G202" t="inlineStr"/>
       <c r="H202" t="inlineStr">
         <is>
-          <t>Concordia Office of Research</t>
+          <t>Office of Research</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>Concordia</t>
         </is>
       </c>
     </row>
@@ -6995,6 +7310,11 @@
           <t>Concordia University</t>
         </is>
       </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>Concordia</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -7033,6 +7353,11 @@
           <t>Concordia University</t>
         </is>
       </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>Concordia</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -7068,7 +7393,12 @@
       <c r="G205" t="inlineStr"/>
       <c r="H205" t="inlineStr">
         <is>
-          <t>Concordia Office of Research</t>
+          <t>Office of Research</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>Concordia</t>
         </is>
       </c>
     </row>
@@ -7106,7 +7436,12 @@
       <c r="G206" t="inlineStr"/>
       <c r="H206" t="inlineStr">
         <is>
-          <t>Concordia Office of Research</t>
+          <t>Office of Research</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>Concordia</t>
         </is>
       </c>
     </row>
@@ -7144,7 +7479,12 @@
       <c r="G207" t="inlineStr"/>
       <c r="H207" t="inlineStr">
         <is>
-          <t>Concordia Fine Arts Faculty</t>
+          <t>Fine Arts</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>Concordia</t>
         </is>
       </c>
     </row>
@@ -7182,7 +7522,12 @@
       <c r="G208" t="inlineStr"/>
       <c r="H208" t="inlineStr">
         <is>
-          <t>Concordia Fine Arts-Engineering</t>
+          <t>Fine Arts-Engineering</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>Concordia</t>
         </is>
       </c>
     </row>
@@ -7220,7 +7565,12 @@
       <c r="G209" t="inlineStr"/>
       <c r="H209" t="inlineStr">
         <is>
-          <t>Concordia Fine Arts-Engineering</t>
+          <t>Fine Arts-Engineering</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>Concordia</t>
         </is>
       </c>
     </row>
@@ -7258,7 +7608,12 @@
       <c r="G210" t="inlineStr"/>
       <c r="H210" t="inlineStr">
         <is>
-          <t>Concordia Fine Arts Faculty</t>
+          <t>Fine Arts</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>Concordia</t>
         </is>
       </c>
     </row>
@@ -7291,6 +7646,7 @@
       </c>
       <c r="G211" t="inlineStr"/>
       <c r="H211" t="inlineStr"/>
+      <c r="I211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -7321,6 +7677,7 @@
       </c>
       <c r="G212" t="inlineStr"/>
       <c r="H212" t="inlineStr"/>
+      <c r="I212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -7351,6 +7708,7 @@
       </c>
       <c r="G213" t="inlineStr"/>
       <c r="H213" t="inlineStr"/>
+      <c r="I213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -7381,6 +7739,7 @@
       </c>
       <c r="G214" t="inlineStr"/>
       <c r="H214" t="inlineStr"/>
+      <c r="I214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -7411,6 +7770,7 @@
       </c>
       <c r="G215" t="inlineStr"/>
       <c r="H215" t="inlineStr"/>
+      <c r="I215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -7441,6 +7801,7 @@
       </c>
       <c r="G216" t="inlineStr"/>
       <c r="H216" t="inlineStr"/>
+      <c r="I216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -7471,6 +7832,7 @@
       </c>
       <c r="G217" t="inlineStr"/>
       <c r="H217" t="inlineStr"/>
+      <c r="I217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -7501,6 +7863,7 @@
       </c>
       <c r="G218" t="inlineStr"/>
       <c r="H218" t="inlineStr"/>
+      <c r="I218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -7531,6 +7894,7 @@
       </c>
       <c r="G219" t="inlineStr"/>
       <c r="H219" t="inlineStr"/>
+      <c r="I219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -7561,6 +7925,7 @@
       </c>
       <c r="G220" t="inlineStr"/>
       <c r="H220" t="inlineStr"/>
+      <c r="I220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -7591,6 +7956,7 @@
       </c>
       <c r="G221" t="inlineStr"/>
       <c r="H221" t="inlineStr"/>
+      <c r="I221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -7621,6 +7987,7 @@
       </c>
       <c r="G222" t="inlineStr"/>
       <c r="H222" t="inlineStr"/>
+      <c r="I222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -7651,6 +8018,7 @@
       </c>
       <c r="G223" t="inlineStr"/>
       <c r="H223" t="inlineStr"/>
+      <c r="I223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -7681,6 +8049,7 @@
       </c>
       <c r="G224" t="inlineStr"/>
       <c r="H224" t="inlineStr"/>
+      <c r="I224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -7711,6 +8080,7 @@
       </c>
       <c r="G225" t="inlineStr"/>
       <c r="H225" t="inlineStr"/>
+      <c r="I225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -7741,6 +8111,7 @@
       </c>
       <c r="G226" t="inlineStr"/>
       <c r="H226" t="inlineStr"/>
+      <c r="I226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -7771,6 +8142,7 @@
       </c>
       <c r="G227" t="inlineStr"/>
       <c r="H227" t="inlineStr"/>
+      <c r="I227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -7801,6 +8173,7 @@
       </c>
       <c r="G228" t="inlineStr"/>
       <c r="H228" t="inlineStr"/>
+      <c r="I228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -7831,6 +8204,7 @@
       </c>
       <c r="G229" t="inlineStr"/>
       <c r="H229" t="inlineStr"/>
+      <c r="I229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -7861,6 +8235,7 @@
       </c>
       <c r="G230" t="inlineStr"/>
       <c r="H230" t="inlineStr"/>
+      <c r="I230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -7891,6 +8266,7 @@
       </c>
       <c r="G231" t="inlineStr"/>
       <c r="H231" t="inlineStr"/>
+      <c r="I231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -7921,6 +8297,7 @@
       </c>
       <c r="G232" t="inlineStr"/>
       <c r="H232" t="inlineStr"/>
+      <c r="I232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -7951,6 +8328,7 @@
       </c>
       <c r="G233" t="inlineStr"/>
       <c r="H233" t="inlineStr"/>
+      <c r="I233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -7981,6 +8359,7 @@
       </c>
       <c r="G234" t="inlineStr"/>
       <c r="H234" t="inlineStr"/>
+      <c r="I234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -8011,6 +8390,7 @@
       </c>
       <c r="G235" t="inlineStr"/>
       <c r="H235" t="inlineStr"/>
+      <c r="I235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -8041,6 +8421,7 @@
       </c>
       <c r="G236" t="inlineStr"/>
       <c r="H236" t="inlineStr"/>
+      <c r="I236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -8071,6 +8452,7 @@
       </c>
       <c r="G237" t="inlineStr"/>
       <c r="H237" t="inlineStr"/>
+      <c r="I237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -8101,6 +8483,7 @@
       </c>
       <c r="G238" t="inlineStr"/>
       <c r="H238" t="inlineStr"/>
+      <c r="I238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -8131,6 +8514,7 @@
       </c>
       <c r="G239" t="inlineStr"/>
       <c r="H239" t="inlineStr"/>
+      <c r="I239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -8161,6 +8545,7 @@
       </c>
       <c r="G240" t="inlineStr"/>
       <c r="H240" t="inlineStr"/>
+      <c r="I240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -8191,6 +8576,7 @@
       </c>
       <c r="G241" t="inlineStr"/>
       <c r="H241" t="inlineStr"/>
+      <c r="I241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -8221,6 +8607,7 @@
       </c>
       <c r="G242" t="inlineStr"/>
       <c r="H242" t="inlineStr"/>
+      <c r="I242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -8251,6 +8638,7 @@
       </c>
       <c r="G243" t="inlineStr"/>
       <c r="H243" t="inlineStr"/>
+      <c r="I243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -8281,6 +8669,7 @@
       </c>
       <c r="G244" t="inlineStr"/>
       <c r="H244" t="inlineStr"/>
+      <c r="I244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -8311,6 +8700,7 @@
       </c>
       <c r="G245" t="inlineStr"/>
       <c r="H245" t="inlineStr"/>
+      <c r="I245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -8341,6 +8731,7 @@
       </c>
       <c r="G246" t="inlineStr"/>
       <c r="H246" t="inlineStr"/>
+      <c r="I246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -8371,6 +8762,7 @@
       </c>
       <c r="G247" t="inlineStr"/>
       <c r="H247" t="inlineStr"/>
+      <c r="I247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -8401,6 +8793,7 @@
       </c>
       <c r="G248" t="inlineStr"/>
       <c r="H248" t="inlineStr"/>
+      <c r="I248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -8431,6 +8824,7 @@
       </c>
       <c r="G249" t="inlineStr"/>
       <c r="H249" t="inlineStr"/>
+      <c r="I249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -8461,6 +8855,7 @@
       </c>
       <c r="G250" t="inlineStr"/>
       <c r="H250" t="inlineStr"/>
+      <c r="I250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -8491,6 +8886,7 @@
       </c>
       <c r="G251" t="inlineStr"/>
       <c r="H251" t="inlineStr"/>
+      <c r="I251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -8521,6 +8917,7 @@
       </c>
       <c r="G252" t="inlineStr"/>
       <c r="H252" t="inlineStr"/>
+      <c r="I252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -8551,6 +8948,7 @@
       </c>
       <c r="G253" t="inlineStr"/>
       <c r="H253" t="inlineStr"/>
+      <c r="I253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -8581,6 +8979,7 @@
       </c>
       <c r="G254" t="inlineStr"/>
       <c r="H254" t="inlineStr"/>
+      <c r="I254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -8611,6 +9010,7 @@
       </c>
       <c r="G255" t="inlineStr"/>
       <c r="H255" t="inlineStr"/>
+      <c r="I255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -8641,6 +9041,7 @@
       </c>
       <c r="G256" t="inlineStr"/>
       <c r="H256" t="inlineStr"/>
+      <c r="I256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -8671,6 +9072,7 @@
       </c>
       <c r="G257" t="inlineStr"/>
       <c r="H257" t="inlineStr"/>
+      <c r="I257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -8701,6 +9103,7 @@
       </c>
       <c r="G258" t="inlineStr"/>
       <c r="H258" t="inlineStr"/>
+      <c r="I258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -8731,6 +9134,7 @@
       </c>
       <c r="G259" t="inlineStr"/>
       <c r="H259" t="inlineStr"/>
+      <c r="I259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -8761,6 +9165,7 @@
       </c>
       <c r="G260" t="inlineStr"/>
       <c r="H260" t="inlineStr"/>
+      <c r="I260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -8791,6 +9196,7 @@
       </c>
       <c r="G261" t="inlineStr"/>
       <c r="H261" t="inlineStr"/>
+      <c r="I261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -8821,6 +9227,7 @@
       </c>
       <c r="G262" t="inlineStr"/>
       <c r="H262" t="inlineStr"/>
+      <c r="I262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -8851,6 +9258,7 @@
       </c>
       <c r="G263" t="inlineStr"/>
       <c r="H263" t="inlineStr"/>
+      <c r="I263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -8881,6 +9289,7 @@
       </c>
       <c r="G264" t="inlineStr"/>
       <c r="H264" t="inlineStr"/>
+      <c r="I264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -8911,6 +9320,7 @@
       </c>
       <c r="G265" t="inlineStr"/>
       <c r="H265" t="inlineStr"/>
+      <c r="I265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -8941,6 +9351,7 @@
       </c>
       <c r="G266" t="inlineStr"/>
       <c r="H266" t="inlineStr"/>
+      <c r="I266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -8971,6 +9382,7 @@
       </c>
       <c r="G267" t="inlineStr"/>
       <c r="H267" t="inlineStr"/>
+      <c r="I267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -9001,6 +9413,7 @@
       </c>
       <c r="G268" t="inlineStr"/>
       <c r="H268" t="inlineStr"/>
+      <c r="I268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -9031,6 +9444,7 @@
       </c>
       <c r="G269" t="inlineStr"/>
       <c r="H269" t="inlineStr"/>
+      <c r="I269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -9061,6 +9475,7 @@
       </c>
       <c r="G270" t="inlineStr"/>
       <c r="H270" t="inlineStr"/>
+      <c r="I270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -9091,6 +9506,7 @@
       </c>
       <c r="G271" t="inlineStr"/>
       <c r="H271" t="inlineStr"/>
+      <c r="I271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -9121,6 +9537,7 @@
       </c>
       <c r="G272" t="inlineStr"/>
       <c r="H272" t="inlineStr"/>
+      <c r="I272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -9151,6 +9568,7 @@
       </c>
       <c r="G273" t="inlineStr"/>
       <c r="H273" t="inlineStr"/>
+      <c r="I273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -9181,6 +9599,7 @@
       </c>
       <c r="G274" t="inlineStr"/>
       <c r="H274" t="inlineStr"/>
+      <c r="I274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -9211,6 +9630,7 @@
       </c>
       <c r="G275" t="inlineStr"/>
       <c r="H275" t="inlineStr"/>
+      <c r="I275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -9241,6 +9661,7 @@
       </c>
       <c r="G276" t="inlineStr"/>
       <c r="H276" t="inlineStr"/>
+      <c r="I276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -9271,6 +9692,7 @@
       </c>
       <c r="G277" t="inlineStr"/>
       <c r="H277" t="inlineStr"/>
+      <c r="I277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -9301,6 +9723,7 @@
       </c>
       <c r="G278" t="inlineStr"/>
       <c r="H278" t="inlineStr"/>
+      <c r="I278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -9331,6 +9754,7 @@
       </c>
       <c r="G279" t="inlineStr"/>
       <c r="H279" t="inlineStr"/>
+      <c r="I279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -9361,6 +9785,7 @@
       </c>
       <c r="G280" t="inlineStr"/>
       <c r="H280" t="inlineStr"/>
+      <c r="I280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -9391,6 +9816,7 @@
       </c>
       <c r="G281" t="inlineStr"/>
       <c r="H281" t="inlineStr"/>
+      <c r="I281" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -9417,6 +9843,7 @@
       </c>
       <c r="G282" t="inlineStr"/>
       <c r="H282" t="inlineStr"/>
+      <c r="I282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -9443,6 +9870,7 @@
       </c>
       <c r="G283" t="inlineStr"/>
       <c r="H283" t="inlineStr"/>
+      <c r="I283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -9469,6 +9897,7 @@
       </c>
       <c r="G284" t="inlineStr"/>
       <c r="H284" t="inlineStr"/>
+      <c r="I284" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -9495,6 +9924,7 @@
       </c>
       <c r="G285" t="inlineStr"/>
       <c r="H285" t="inlineStr"/>
+      <c r="I285" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -9525,6 +9955,7 @@
       </c>
       <c r="G286" t="inlineStr"/>
       <c r="H286" t="inlineStr"/>
+      <c r="I286" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Supervision headlines: degree + name (+ qualifier), strip Supervisor label
'PhD Supervisor: X' → 'PhD X'
'PhD Secondary Supervisor: X' → 'PhD X (Secondary)'
'PhD Co-supervisor: X' → 'PhD X (Co-supervisor)'
'PhD Committee Member: X' → 'PhD X (Committee)'
Same pattern for Masters, Postdoc, Undergraduate, Grad Certificate.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/cv-data/cv.xlsx
+++ b/data/cv-data/cv.xlsx
@@ -15457,7 +15457,7 @@
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>Undergraduate Honours Supervisor: [Student A]</t>
+          <t>Undergraduate [Student A] (Honours)</t>
         </is>
       </c>
       <c r="D407" t="inlineStr">
@@ -15493,7 +15493,7 @@
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>Undergraduate Honours Supervisor: [Student B]</t>
+          <t>Undergraduate [Student B] (Honours)</t>
         </is>
       </c>
       <c r="D408" t="inlineStr">
@@ -15529,7 +15529,7 @@
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>Undergraduate Independent Study: [Student C]</t>
+          <t>Undergraduate [Student C] (Independent Study)</t>
         </is>
       </c>
       <c r="D409" t="inlineStr">
@@ -15565,7 +15565,7 @@
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>Graduate Certificate Supervisor: [Student D]</t>
+          <t>Grad Certificate [Student D]</t>
         </is>
       </c>
       <c r="D410" t="inlineStr">
@@ -15601,7 +15601,7 @@
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>Graduate Certificate Supervisor: [Student E]</t>
+          <t>Grad Certificate [Student E]</t>
         </is>
       </c>
       <c r="D411" t="inlineStr">
@@ -15637,7 +15637,7 @@
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>Masters Supervisor: Vanessa Racine</t>
+          <t>Masters Vanessa Racine</t>
         </is>
       </c>
       <c r="D412" t="inlineStr">
@@ -15673,7 +15673,7 @@
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>Masters Committee: Tarcisio Cataldi Tegani</t>
+          <t>Masters Tarcisio Cataldi Tegani (Committee)</t>
         </is>
       </c>
       <c r="D413" t="inlineStr">
@@ -15709,7 +15709,7 @@
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>Masters Supervisor: Caeleigh Lightning Long</t>
+          <t>Masters Caeleigh Lightning Long</t>
         </is>
       </c>
       <c r="D414" t="inlineStr">
@@ -15745,7 +15745,7 @@
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>Masters Supervisor: Sébastien Aubin</t>
+          <t>Masters Sébastien Aubin</t>
         </is>
       </c>
       <c r="D415" t="inlineStr">
@@ -15781,7 +15781,7 @@
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>Masters Supervisor: Waylon Wilson</t>
+          <t>Masters Waylon Wilson</t>
         </is>
       </c>
       <c r="D416" t="inlineStr">
@@ -15817,7 +15817,7 @@
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>Masters Supervisor: Maize Longboat</t>
+          <t>Masters Maize Longboat</t>
         </is>
       </c>
       <c r="D417" t="inlineStr">
@@ -15853,7 +15853,7 @@
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>Masters Co-supervisor: Nicholas Gwyn Shulman</t>
+          <t>Masters Nicholas Gwyn Shulman (Co-supervisor)</t>
         </is>
       </c>
       <c r="D418" t="inlineStr">
@@ -15889,7 +15889,7 @@
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>Masters Supervisor: Morgan Kennedy</t>
+          <t>Masters Morgan Kennedy</t>
         </is>
       </c>
       <c r="D419" t="inlineStr">
@@ -15925,7 +15925,7 @@
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>Masters Co-supervisor: Nikolaos Chandolias</t>
+          <t>Masters Nikolaos Chandolias (Co-supervisor)</t>
         </is>
       </c>
       <c r="D420" t="inlineStr">
@@ -15961,7 +15961,7 @@
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>Masters Supervisor: Leslie Plumb</t>
+          <t>Masters Leslie Plumb</t>
         </is>
       </c>
       <c r="D421" t="inlineStr">
@@ -15997,7 +15997,7 @@
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>Masters Co-supervisor: Mia Song</t>
+          <t>Masters Mia Song (Co-supervisor)</t>
         </is>
       </c>
       <c r="D422" t="inlineStr">
@@ -16033,7 +16033,7 @@
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>Masters Committee: Rozita Naghshin</t>
+          <t>Masters Rozita Naghshin (Committee)</t>
         </is>
       </c>
       <c r="D423" t="inlineStr">
@@ -16069,7 +16069,7 @@
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>PhD Supervisor: Juliet Mackie</t>
+          <t>PhD Juliet Mackie</t>
         </is>
       </c>
       <c r="D424" t="inlineStr">
@@ -16105,7 +16105,7 @@
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>PhD Supervisor: Mel Lefebvre</t>
+          <t>PhD Mel Lefebvre</t>
         </is>
       </c>
       <c r="D425" t="inlineStr">
@@ -16141,7 +16141,7 @@
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>PhD Co-supervisor: Jessica Barudin</t>
+          <t>PhD Jessica Barudin (Co-supervisor)</t>
         </is>
       </c>
       <c r="D426" t="inlineStr">
@@ -16177,7 +16177,7 @@
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>PhD Supervisor: Suzanne Kite</t>
+          <t>PhD Suzanne Kite</t>
         </is>
       </c>
       <c r="D427" t="inlineStr">
@@ -16213,7 +16213,7 @@
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>PhD Secondary Supervisor: Nafisa Sarwath</t>
+          <t>PhD Nafisa Sarwath (Secondary)</t>
         </is>
       </c>
       <c r="D428" t="inlineStr">
@@ -16249,7 +16249,7 @@
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>PhD Secondary Supervisor: Michelle Brown</t>
+          <t>PhD Michelle Brown (Secondary)</t>
         </is>
       </c>
       <c r="D429" t="inlineStr">
@@ -16285,7 +16285,7 @@
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>PhD Co-supervisor: Elizabeth LaPensée</t>
+          <t>PhD Elizabeth LaPensée (Co-supervisor)</t>
         </is>
       </c>
       <c r="D430" t="inlineStr">
@@ -16321,7 +16321,7 @@
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>PhD Secondary Supervisor: Miao Song</t>
+          <t>PhD Miao Song (Secondary)</t>
         </is>
       </c>
       <c r="D431" t="inlineStr">
@@ -16357,7 +16357,7 @@
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>PhD Secondary Supervisor: David Johnston</t>
+          <t>PhD David Johnston (Secondary)</t>
         </is>
       </c>
       <c r="D432" t="inlineStr">
@@ -16393,7 +16393,7 @@
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t>PhD Committee Member: Rozita Naghshin</t>
+          <t>PhD Rozita Naghshin (Committee)</t>
         </is>
       </c>
       <c r="D433" t="inlineStr">
@@ -16429,7 +16429,7 @@
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t>Postdoctoral Fellow: Melemaikalani Moniz</t>
+          <t>Postdoc Melemaikalani Moniz</t>
         </is>
       </c>
       <c r="D434" t="inlineStr">
@@ -16465,7 +16465,7 @@
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>Postdoctoral Fellow: Ceyda Yolgörmez</t>
+          <t>Postdoc Ceyda Yolgörmez</t>
         </is>
       </c>
       <c r="D435" t="inlineStr">
@@ -16501,7 +16501,7 @@
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>Postdoctoral Fellow: Leuli Eschraghi</t>
+          <t>Postdoc Leuli Eschraghi</t>
         </is>
       </c>
       <c r="D436" t="inlineStr">

</xml_diff>

<commit_message>
Supervision headlines: drop degree-level prefix (redundant with category band)
'PhD Suzanne Kite' → 'Suzanne Kite'
'Miao Song (Secondary)', 'Rozita Naghshin (Committee)', etc. unchanged otherwise.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/cv-data/cv.xlsx
+++ b/data/cv-data/cv.xlsx
@@ -15457,7 +15457,7 @@
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>Undergraduate [Student A] (Honours)</t>
+          <t>[Student A] (Honours)</t>
         </is>
       </c>
       <c r="D407" t="inlineStr">
@@ -15493,7 +15493,7 @@
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>Undergraduate [Student B] (Honours)</t>
+          <t>[Student B] (Honours)</t>
         </is>
       </c>
       <c r="D408" t="inlineStr">
@@ -15529,7 +15529,7 @@
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>Undergraduate [Student C] (Independent Study)</t>
+          <t>[Student C] (Independent Study)</t>
         </is>
       </c>
       <c r="D409" t="inlineStr">
@@ -15565,7 +15565,7 @@
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>Grad Certificate [Student D]</t>
+          <t>[Student D]</t>
         </is>
       </c>
       <c r="D410" t="inlineStr">
@@ -15601,7 +15601,7 @@
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>Grad Certificate [Student E]</t>
+          <t>[Student E]</t>
         </is>
       </c>
       <c r="D411" t="inlineStr">
@@ -15637,7 +15637,7 @@
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>Masters Vanessa Racine</t>
+          <t>Vanessa Racine</t>
         </is>
       </c>
       <c r="D412" t="inlineStr">
@@ -15673,7 +15673,7 @@
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>Masters Tarcisio Cataldi Tegani (Committee)</t>
+          <t>Tarcisio Cataldi Tegani (Committee)</t>
         </is>
       </c>
       <c r="D413" t="inlineStr">
@@ -15709,7 +15709,7 @@
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>Masters Caeleigh Lightning Long</t>
+          <t>Caeleigh Lightning Long</t>
         </is>
       </c>
       <c r="D414" t="inlineStr">
@@ -15745,7 +15745,7 @@
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>Masters Sébastien Aubin</t>
+          <t>Sébastien Aubin</t>
         </is>
       </c>
       <c r="D415" t="inlineStr">
@@ -15781,7 +15781,7 @@
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>Masters Waylon Wilson</t>
+          <t>Waylon Wilson</t>
         </is>
       </c>
       <c r="D416" t="inlineStr">
@@ -15817,7 +15817,7 @@
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>Masters Maize Longboat</t>
+          <t>Maize Longboat</t>
         </is>
       </c>
       <c r="D417" t="inlineStr">
@@ -15853,7 +15853,7 @@
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>Masters Nicholas Gwyn Shulman (Co-supervisor)</t>
+          <t>Nicholas Gwyn Shulman (Co-supervisor)</t>
         </is>
       </c>
       <c r="D418" t="inlineStr">
@@ -15889,7 +15889,7 @@
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>Masters Morgan Kennedy</t>
+          <t>Morgan Kennedy</t>
         </is>
       </c>
       <c r="D419" t="inlineStr">
@@ -15925,7 +15925,7 @@
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>Masters Nikolaos Chandolias (Co-supervisor)</t>
+          <t>Nikolaos Chandolias (Co-supervisor)</t>
         </is>
       </c>
       <c r="D420" t="inlineStr">
@@ -15961,7 +15961,7 @@
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>Masters Leslie Plumb</t>
+          <t>Leslie Plumb</t>
         </is>
       </c>
       <c r="D421" t="inlineStr">
@@ -15997,7 +15997,7 @@
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>Masters Mia Song (Co-supervisor)</t>
+          <t>Mia Song (Co-supervisor)</t>
         </is>
       </c>
       <c r="D422" t="inlineStr">
@@ -16033,7 +16033,7 @@
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>Masters Rozita Naghshin (Committee)</t>
+          <t>Rozita Naghshin (Committee)</t>
         </is>
       </c>
       <c r="D423" t="inlineStr">
@@ -16069,7 +16069,7 @@
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>PhD Juliet Mackie</t>
+          <t>Juliet Mackie</t>
         </is>
       </c>
       <c r="D424" t="inlineStr">
@@ -16105,7 +16105,7 @@
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>PhD Mel Lefebvre</t>
+          <t>Mel Lefebvre</t>
         </is>
       </c>
       <c r="D425" t="inlineStr">
@@ -16141,7 +16141,7 @@
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>PhD Jessica Barudin (Co-supervisor)</t>
+          <t>Jessica Barudin (Co-supervisor)</t>
         </is>
       </c>
       <c r="D426" t="inlineStr">
@@ -16177,7 +16177,7 @@
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>PhD Suzanne Kite</t>
+          <t>Suzanne Kite</t>
         </is>
       </c>
       <c r="D427" t="inlineStr">
@@ -16213,7 +16213,7 @@
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>PhD Nafisa Sarwath (Secondary)</t>
+          <t>Nafisa Sarwath (Secondary)</t>
         </is>
       </c>
       <c r="D428" t="inlineStr">
@@ -16249,7 +16249,7 @@
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>PhD Michelle Brown (Secondary)</t>
+          <t>Michelle Brown (Secondary)</t>
         </is>
       </c>
       <c r="D429" t="inlineStr">
@@ -16285,7 +16285,7 @@
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>PhD Elizabeth LaPensée (Co-supervisor)</t>
+          <t>Elizabeth LaPensée (Co-supervisor)</t>
         </is>
       </c>
       <c r="D430" t="inlineStr">
@@ -16321,7 +16321,7 @@
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>PhD Miao Song (Secondary)</t>
+          <t>Miao Song (Secondary)</t>
         </is>
       </c>
       <c r="D431" t="inlineStr">
@@ -16357,7 +16357,7 @@
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>PhD David Johnston (Secondary)</t>
+          <t>David Johnston (Secondary)</t>
         </is>
       </c>
       <c r="D432" t="inlineStr">
@@ -16393,7 +16393,7 @@
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t>PhD Rozita Naghshin (Committee)</t>
+          <t>Rozita Naghshin (Committee)</t>
         </is>
       </c>
       <c r="D433" t="inlineStr">
@@ -16429,7 +16429,7 @@
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t>Postdoc Melemaikalani Moniz</t>
+          <t>Melemaikalani Moniz</t>
         </is>
       </c>
       <c r="D434" t="inlineStr">
@@ -16465,7 +16465,7 @@
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>Postdoc Ceyda Yolgörmez</t>
+          <t>Ceyda Yolgörmez</t>
         </is>
       </c>
       <c r="D435" t="inlineStr">
@@ -16501,7 +16501,7 @@
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>Postdoc Leuli Eschraghi</t>
+          <t>Leuli Eschraghi</t>
         </is>
       </c>
       <c r="D436" t="inlineStr">

</xml_diff>

<commit_message>
Grad Certificate: replace synthetic placeholders with 12 real students
Sourced from Teaching & Service Google Doc. Adriana Navarro Sainz
through Justyna Latek (2002–2015), with thesis titles where available.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/cv-data/cv.xlsx
+++ b/data/cv-data/cv.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J458"/>
+  <dimension ref="A1:J468"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15555,22 +15555,22 @@
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>01/01/2023</t>
+          <t>01/01/2014</t>
         </is>
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>12/31/2024</t>
+          <t>12/31/2015</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>[Student D]</t>
+          <t>Adriana Navarro Sainz</t>
         </is>
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>SYNTHETIC. Graduate certificate in computation arts. Concordia University.</t>
+          <t>Concordia University.</t>
         </is>
       </c>
       <c r="E410" t="inlineStr"/>
@@ -15591,22 +15591,22 @@
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>01/01/2021</t>
+          <t>01/01/2014</t>
         </is>
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>12/31/2022</t>
+          <t>12/31/2015</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>[Student E]</t>
+          <t>Guillaume Bourdon</t>
         </is>
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>SYNTHETIC. Graduate certificate in digital fabrication and Indigenous design. Concordia University.</t>
+          <t>Concordia University.</t>
         </is>
       </c>
       <c r="E411" t="inlineStr"/>
@@ -15627,28 +15627,28 @@
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>01/01/2022</t>
+          <t>01/01/2012</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>02/25/2026</t>
+          <t>12/31/2013</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>Vanessa Racine</t>
+          <t>Joanna Pederson</t>
         </is>
       </c>
       <c r="D412" t="inlineStr">
         <is>
-          <t>Anishinaabe Love: Epistemologies &amp; Videogames. Concordia University.</t>
+          <t>Augmented Reality: Save the Ghost Signs. Concordia University.</t>
         </is>
       </c>
       <c r="E412" t="inlineStr"/>
       <c r="F412" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Grad Certificate</t>
         </is>
       </c>
       <c r="G412" t="inlineStr"/>
@@ -15663,28 +15663,28 @@
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>01/01/2022</t>
+          <t>01/01/2010</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>12/31/2025</t>
+          <t>12/31/2011</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>Tarcisio Cataldi Tegani (Committee)</t>
+          <t>Phil Lichti</t>
         </is>
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>Speculative Vexillology: Exploring National Identity and Imagining Afro-Brazilian Futures through Flags. Concordia University.</t>
+          <t>The Soundwalk as Documentary Practice. Concordia University.</t>
         </is>
       </c>
       <c r="E413" t="inlineStr"/>
       <c r="F413" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Grad Certificate</t>
         </is>
       </c>
       <c r="G413" t="inlineStr"/>
@@ -15699,28 +15699,28 @@
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>01/01/2021</t>
+          <t>01/01/2010</t>
         </is>
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>12/31/2024</t>
+          <t>12/31/2011</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>Caeleigh Lightning Long</t>
+          <t>Santiago Salciado</t>
         </is>
       </c>
       <c r="D414" t="inlineStr">
         <is>
-          <t>Wawêsiwîn: The Act of Dressing Up — A Research Cree-ation Project. Concordia University.</t>
+          <t>Improving the Design Process for Textbooks. Concordia University.</t>
         </is>
       </c>
       <c r="E414" t="inlineStr"/>
       <c r="F414" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Grad Certificate</t>
         </is>
       </c>
       <c r="G414" t="inlineStr"/>
@@ -15735,28 +15735,28 @@
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>01/01/2018</t>
+          <t>01/01/2006</t>
         </is>
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>12/31/2023</t>
+          <t>12/31/2007</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>Sébastien Aubin</t>
+          <t>Oliver Tsuji</t>
         </is>
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>Designing Culturally Grounded Cree Syllabaries. Concordia University.</t>
+          <t>Narrative in Digital Media. Concordia University.</t>
         </is>
       </c>
       <c r="E415" t="inlineStr"/>
       <c r="F415" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Grad Certificate</t>
         </is>
       </c>
       <c r="G415" t="inlineStr"/>
@@ -15771,28 +15771,28 @@
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>01/01/2018</t>
+          <t>01/01/2005</t>
         </is>
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>12/31/2021</t>
+          <t>12/31/2006</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>Waylon Wilson</t>
+          <t>Louis Goupille</t>
         </is>
       </c>
       <c r="D416" t="inlineStr">
         <is>
-          <t>Tuscarora Virtual Realities. Concordia University.</t>
+          <t>Painterly Approaches to Virtual Environments. Concordia University.</t>
         </is>
       </c>
       <c r="E416" t="inlineStr"/>
       <c r="F416" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Grad Certificate</t>
         </is>
       </c>
       <c r="G416" t="inlineStr"/>
@@ -15807,28 +15807,28 @@
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>01/01/2017</t>
+          <t>01/01/2005</t>
         </is>
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>12/31/2019</t>
+          <t>12/31/2006</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>Maize Longboat</t>
+          <t>Thibaut Duverneix</t>
         </is>
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>Haudenosaunee Storytelling via Video Games. Concordia University.</t>
+          <t>Concordia University.</t>
         </is>
       </c>
       <c r="E417" t="inlineStr"/>
       <c r="F417" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Grad Certificate</t>
         </is>
       </c>
       <c r="G417" t="inlineStr"/>
@@ -15843,28 +15843,28 @@
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>01/01/2016</t>
+          <t>01/01/2003</t>
         </is>
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>12/31/2020</t>
+          <t>12/31/2004</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>Nicholas Gwyn Shulman (Co-supervisor)</t>
+          <t>Farah Jamaluddin</t>
         </is>
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>Network Arts: Seeing and Making Network Organisms. Concordia University.</t>
+          <t>Concordia University.</t>
         </is>
       </c>
       <c r="E418" t="inlineStr"/>
       <c r="F418" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Grad Certificate</t>
         </is>
       </c>
       <c r="G418" t="inlineStr"/>
@@ -15879,28 +15879,28 @@
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>01/01/2014</t>
+          <t>01/01/2003</t>
         </is>
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>12/31/2024</t>
+          <t>12/31/2005</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>Morgan Kennedy</t>
+          <t>Dalia Radwan</t>
         </is>
       </c>
       <c r="D419" t="inlineStr">
         <is>
-          <t>Storied Indigeneity in Videogames: Post-Indian Warriors and Indie Japan. Concordia University.</t>
+          <t>Concordia University.</t>
         </is>
       </c>
       <c r="E419" t="inlineStr"/>
       <c r="F419" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Grad Certificate</t>
         </is>
       </c>
       <c r="G419" t="inlineStr"/>
@@ -15915,28 +15915,28 @@
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>01/01/2012</t>
+          <t>01/01/2002</t>
         </is>
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>12/31/2015</t>
+          <t>12/31/2003</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>Nikolaos Chandolias (Co-supervisor)</t>
+          <t>John Stuart</t>
         </is>
       </c>
       <c r="D420" t="inlineStr">
         <is>
-          <t>KinectEcho: Gesture and Vocal Recognition in New Media, Interactive Art and Live Events. Concordia University.</t>
+          <t>Concordia University.</t>
         </is>
       </c>
       <c r="E420" t="inlineStr"/>
       <c r="F420" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Grad Certificate</t>
         </is>
       </c>
       <c r="G420" t="inlineStr"/>
@@ -15951,28 +15951,28 @@
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>01/01/2006</t>
+          <t>01/01/2002</t>
         </is>
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>12/31/2007</t>
+          <t>12/31/2003</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>Leslie Plumb</t>
+          <t>Justyna Latek</t>
         </is>
       </c>
       <c r="D421" t="inlineStr">
         <is>
-          <t>Transversal Entanglements: Research-Creation and the Design Process for Inflexions. Concordia University.</t>
+          <t>Concordia University.</t>
         </is>
       </c>
       <c r="E421" t="inlineStr"/>
       <c r="F421" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Grad Certificate</t>
         </is>
       </c>
       <c r="G421" t="inlineStr"/>
@@ -15987,22 +15987,22 @@
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>01/01/2004</t>
+          <t>01/01/2022</t>
         </is>
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>12/31/2008</t>
+          <t>02/25/2026</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>Mia Song (Co-supervisor)</t>
+          <t>Vanessa Racine</t>
         </is>
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>Computer-Assisted Interactive Documentary and Performance Arts in Illimitable Space. Concordia University.</t>
+          <t>Anishinaabe Love: Epistemologies &amp; Videogames. Concordia University.</t>
         </is>
       </c>
       <c r="E422" t="inlineStr"/>
@@ -16023,22 +16023,22 @@
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>01/01/2003</t>
+          <t>01/01/2022</t>
         </is>
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>12/31/2005</t>
+          <t>12/31/2025</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>Rozita Naghshin (Committee)</t>
+          <t>Tarcisio Cataldi Tegani (Committee)</t>
         </is>
       </c>
       <c r="D423" t="inlineStr">
         <is>
-          <t>CASE Tool Simplification Via Task-Sensitive Metaphor. Concordia University.</t>
+          <t>Speculative Vexillology: Exploring National Identity and Imagining Afro-Brazilian Futures through Flags. Concordia University.</t>
         </is>
       </c>
       <c r="E423" t="inlineStr"/>
@@ -16059,28 +16059,28 @@
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>01/01/2023</t>
+          <t>01/01/2021</t>
         </is>
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>02/25/2026</t>
+          <t>12/31/2024</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>Juliet Mackie</t>
+          <t>Caeleigh Lightning Long</t>
         </is>
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>Reconstituting Indigenous Identities through Portraiture and Storytelling. Concordia University.</t>
+          <t>Wawêsiwîn: The Act of Dressing Up — A Research Cree-ation Project. Concordia University.</t>
         </is>
       </c>
       <c r="E424" t="inlineStr"/>
       <c r="F424" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="G424" t="inlineStr"/>
@@ -16095,28 +16095,28 @@
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>01/01/2021</t>
+          <t>01/01/2018</t>
         </is>
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>12/31/2024</t>
+          <t>12/31/2023</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>Mel Lefebvre</t>
+          <t>Sébastien Aubin</t>
         </is>
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t>Healing Through Ancestral Skin Marking: Traditional Tattooing as Healing and (Re)connection for Indigenous People. Concordia University.</t>
+          <t>Designing Culturally Grounded Cree Syllabaries. Concordia University.</t>
         </is>
       </c>
       <c r="E425" t="inlineStr"/>
       <c r="F425" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="G425" t="inlineStr"/>
@@ -16131,28 +16131,28 @@
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>01/01/2019</t>
+          <t>01/01/2018</t>
         </is>
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>12/31/2023</t>
+          <t>12/31/2021</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>Jessica Barudin (Co-supervisor)</t>
+          <t>Waylon Wilson</t>
         </is>
       </c>
       <c r="D426" t="inlineStr">
         <is>
-          <t>Re-connecting Through Women's Teachings, Language and Movement. Concordia University.</t>
+          <t>Tuscarora Virtual Realities. Concordia University.</t>
         </is>
       </c>
       <c r="E426" t="inlineStr"/>
       <c r="F426" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="G426" t="inlineStr"/>
@@ -16172,23 +16172,23 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>12/31/2023</t>
+          <t>12/31/2019</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>Suzanne Kite</t>
+          <t>Maize Longboat</t>
         </is>
       </c>
       <c r="D427" t="inlineStr">
         <is>
-          <t>Lakota Epistemology, Performance Practice, and Digital Technology. Concordia University.</t>
+          <t>Haudenosaunee Storytelling via Video Games. Concordia University.</t>
         </is>
       </c>
       <c r="E427" t="inlineStr"/>
       <c r="F427" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="G427" t="inlineStr"/>
@@ -16203,28 +16203,28 @@
     <row r="428">
       <c r="A428" t="inlineStr">
         <is>
-          <t>01/01/2017</t>
+          <t>01/01/2016</t>
         </is>
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>02/25/2026</t>
+          <t>12/31/2020</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>Nafisa Sarwath (Secondary)</t>
+          <t>Nicholas Gwyn Shulman (Co-supervisor)</t>
         </is>
       </c>
       <c r="D428" t="inlineStr">
         <is>
-          <t>Indigenous knowledge, resilience and adaptive capacity. Concordia University.</t>
+          <t>Network Arts: Seeing and Making Network Organisms. Concordia University.</t>
         </is>
       </c>
       <c r="E428" t="inlineStr"/>
       <c r="F428" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="G428" t="inlineStr"/>
@@ -16239,28 +16239,28 @@
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>01/01/2016</t>
+          <t>01/01/2014</t>
         </is>
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>12/31/2021</t>
+          <t>12/31/2024</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>Michelle Brown (Secondary)</t>
+          <t>Morgan Kennedy</t>
         </is>
       </c>
       <c r="D429" t="inlineStr">
         <is>
-          <t>(Re)Coding Resurgence: Indigenous Digital Media Kinnections. University of Hawaii Mānoa.</t>
+          <t>Storied Indigeneity in Videogames: Post-Indian Warriors and Indie Japan. Concordia University.</t>
         </is>
       </c>
       <c r="E429" t="inlineStr"/>
       <c r="F429" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="G429" t="inlineStr"/>
@@ -16275,28 +16275,28 @@
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>01/01/2007</t>
+          <t>01/01/2012</t>
         </is>
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>12/31/2014</t>
+          <t>12/31/2015</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>Elizabeth LaPensée (Co-supervisor)</t>
+          <t>Nikolaos Chandolias (Co-supervisor)</t>
         </is>
       </c>
       <c r="D430" t="inlineStr">
         <is>
-          <t>Experiencing Stories: Narrative and Experience in Interactive Media. Simon Fraser University.</t>
+          <t>KinectEcho: Gesture and Vocal Recognition in New Media, Interactive Art and Live Events. Concordia University.</t>
         </is>
       </c>
       <c r="E430" t="inlineStr"/>
       <c r="F430" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="G430" t="inlineStr"/>
@@ -16311,28 +16311,28 @@
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>01/01/2008</t>
+          <t>01/01/2006</t>
         </is>
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>12/31/2012</t>
+          <t>12/31/2007</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>Miao Song (Secondary)</t>
+          <t>Leslie Plumb</t>
         </is>
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t>Experiencing Stories: Narrative and Experience in Interactive Media. Concordia University.</t>
+          <t>Transversal Entanglements: Research-Creation and the Design Process for Inflexions. Concordia University.</t>
         </is>
       </c>
       <c r="E431" t="inlineStr"/>
       <c r="F431" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="G431" t="inlineStr"/>
@@ -16347,28 +16347,28 @@
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>01/01/2008</t>
+          <t>01/01/2004</t>
         </is>
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>12/31/2011</t>
+          <t>12/31/2008</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>David Johnston (Secondary)</t>
+          <t>Mia Song (Co-supervisor)</t>
         </is>
       </c>
       <c r="D432" t="inlineStr">
         <is>
-          <t>Aesthetic Animism: Digital Poetry as Ontological Probe. Concordia University.</t>
+          <t>Computer-Assisted Interactive Documentary and Performance Arts in Illimitable Space. Concordia University.</t>
         </is>
       </c>
       <c r="E432" t="inlineStr"/>
       <c r="F432" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="G432" t="inlineStr"/>
@@ -16383,12 +16383,12 @@
     <row r="433">
       <c r="A433" t="inlineStr">
         <is>
-          <t>01/01/2005</t>
+          <t>01/01/2003</t>
         </is>
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>12/31/2008</t>
+          <t>12/31/2005</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
@@ -16398,13 +16398,13 @@
       </c>
       <c r="D433" t="inlineStr">
         <is>
-          <t>Software Design as an Aesthetic Design Practice. Concordia University.</t>
+          <t>CASE Tool Simplification Via Task-Sensitive Metaphor. Concordia University.</t>
         </is>
       </c>
       <c r="E433" t="inlineStr"/>
       <c r="F433" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="G433" t="inlineStr"/>
@@ -16419,7 +16419,7 @@
     <row r="434">
       <c r="A434" t="inlineStr">
         <is>
-          <t>01/01/2025</t>
+          <t>01/01/2023</t>
         </is>
       </c>
       <c r="B434" t="inlineStr">
@@ -16429,18 +16429,18 @@
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t>Melemaikalani Moniz</t>
+          <t>Juliet Mackie</t>
         </is>
       </c>
       <c r="D434" t="inlineStr">
         <is>
-          <t>Postdoctoral Fellow in Abundant Soils. Concordia University.</t>
+          <t>Reconstituting Indigenous Identities through Portraiture and Storytelling. Concordia University.</t>
         </is>
       </c>
       <c r="E434" t="inlineStr"/>
       <c r="F434" t="inlineStr">
         <is>
-          <t>Postdoc</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="G434" t="inlineStr"/>
@@ -16455,28 +16455,28 @@
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>01/01/2024</t>
+          <t>01/01/2021</t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>12/31/2026</t>
+          <t>12/31/2024</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>Ceyda Yolgörmez</t>
+          <t>Mel Lefebvre</t>
         </is>
       </c>
       <c r="D435" t="inlineStr">
         <is>
-          <t>Horizon Postdoctoral Fellow in Abundant Intelligences. Concordia University.</t>
+          <t>Healing Through Ancestral Skin Marking: Traditional Tattooing as Healing and (Re)connection for Indigenous People. Concordia University.</t>
         </is>
       </c>
       <c r="E435" t="inlineStr"/>
       <c r="F435" t="inlineStr">
         <is>
-          <t>Postdoc</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="G435" t="inlineStr"/>
@@ -16496,23 +16496,23 @@
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>12/31/2021</t>
+          <t>12/31/2023</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>Leuli Eschraghi</t>
+          <t>Jessica Barudin (Co-supervisor)</t>
         </is>
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t>Horizon Postdoctoral Fellow in Indigenous Futures. Concordia University.</t>
+          <t>Re-connecting Through Women's Teachings, Language and Movement. Concordia University.</t>
         </is>
       </c>
       <c r="E436" t="inlineStr"/>
       <c r="F436" t="inlineStr">
         <is>
-          <t>Postdoc</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="G436" t="inlineStr"/>
@@ -16527,130 +16527,146 @@
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>01/01/2010</t>
+          <t>01/01/2017</t>
         </is>
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>12/31/2018</t>
+          <t>12/31/2023</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>Acting Chair</t>
+          <t>Suzanne Kite</t>
         </is>
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>Department of Design and Computation Arts, Concordia University. Various 1-to-2-week terms.</t>
+          <t>Lakota Epistemology, Performance Practice, and Digital Technology. Concordia University.</t>
         </is>
       </c>
       <c r="E437" t="inlineStr"/>
       <c r="F437" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="G437" t="inlineStr"/>
       <c r="H437" t="inlineStr"/>
       <c r="I437" t="inlineStr"/>
-      <c r="J437" t="inlineStr"/>
+      <c r="J437" t="inlineStr">
+        <is>
+          <t>Supervision</t>
+        </is>
+      </c>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
         <is>
-          <t>09/01/2003</t>
+          <t>01/01/2017</t>
         </is>
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>08/31/2013</t>
+          <t>02/25/2026</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>Computation Arts Undergraduate Program Director / Co-director</t>
+          <t>Nafisa Sarwath (Secondary)</t>
         </is>
       </c>
       <c r="D438" t="inlineStr">
         <is>
-          <t>Department of Design and Computation Arts, Concordia University.</t>
+          <t>Indigenous knowledge, resilience and adaptive capacity. Concordia University.</t>
         </is>
       </c>
       <c r="E438" t="inlineStr"/>
       <c r="F438" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="G438" t="inlineStr"/>
       <c r="H438" t="inlineStr"/>
       <c r="I438" t="inlineStr"/>
-      <c r="J438" t="inlineStr"/>
+      <c r="J438" t="inlineStr">
+        <is>
+          <t>Supervision</t>
+        </is>
+      </c>
     </row>
     <row r="439">
       <c r="A439" t="inlineStr">
         <is>
-          <t>09/01/2005</t>
+          <t>01/01/2016</t>
         </is>
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>08/31/2008</t>
+          <t>12/31/2021</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>Graduate Program Director</t>
+          <t>Michelle Brown (Secondary)</t>
         </is>
       </c>
       <c r="D439" t="inlineStr">
         <is>
-          <t>Department of Design and Computation Arts, Concordia University.</t>
+          <t>(Re)Coding Resurgence: Indigenous Digital Media Kinnections. University of Hawaii Mānoa.</t>
         </is>
       </c>
       <c r="E439" t="inlineStr"/>
       <c r="F439" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="G439" t="inlineStr"/>
       <c r="H439" t="inlineStr"/>
       <c r="I439" t="inlineStr"/>
-      <c r="J439" t="inlineStr"/>
+      <c r="J439" t="inlineStr">
+        <is>
+          <t>Supervision</t>
+        </is>
+      </c>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
         <is>
-          <t>09/01/2003</t>
+          <t>01/01/2007</t>
         </is>
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>08/31/2014</t>
+          <t>12/31/2014</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
         <is>
-          <t>Computation Lab Director</t>
+          <t>Elizabeth LaPensée (Co-supervisor)</t>
         </is>
       </c>
       <c r="D440" t="inlineStr">
         <is>
-          <t>Department of Design and Computation Arts, Concordia University.</t>
+          <t>Experiencing Stories: Narrative and Experience in Interactive Media. Simon Fraser University.</t>
         </is>
       </c>
       <c r="E440" t="inlineStr"/>
       <c r="F440" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="G440" t="inlineStr"/>
       <c r="H440" t="inlineStr"/>
       <c r="I440" t="inlineStr"/>
-      <c r="J440" t="inlineStr"/>
+      <c r="J440" t="inlineStr">
+        <is>
+          <t>Supervision</t>
+        </is>
+      </c>
     </row>
     <row r="441">
       <c r="A441" t="inlineStr">
@@ -16660,209 +16676,233 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>12/31/2020</t>
+          <t>12/31/2012</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t>Personnel Committee</t>
+          <t>Miao Song (Secondary)</t>
         </is>
       </c>
       <c r="D441" t="inlineStr">
         <is>
-          <t>Department of Design and Computation Arts, Concordia University.</t>
+          <t>Experiencing Stories: Narrative and Experience in Interactive Media. Concordia University.</t>
         </is>
       </c>
       <c r="E441" t="inlineStr"/>
       <c r="F441" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="G441" t="inlineStr"/>
       <c r="H441" t="inlineStr"/>
       <c r="I441" t="inlineStr"/>
-      <c r="J441" t="inlineStr"/>
+      <c r="J441" t="inlineStr">
+        <is>
+          <t>Supervision</t>
+        </is>
+      </c>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>01/01/2002</t>
+          <t>01/01/2008</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>12/31/2014</t>
+          <t>12/31/2011</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>CART Curriculum Committee, Chair</t>
+          <t>David Johnston (Secondary)</t>
         </is>
       </c>
       <c r="D442" t="inlineStr">
         <is>
-          <t>Department of Design and Computation Arts, Concordia University.</t>
+          <t>Aesthetic Animism: Digital Poetry as Ontological Probe. Concordia University.</t>
         </is>
       </c>
       <c r="E442" t="inlineStr"/>
       <c r="F442" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="G442" t="inlineStr"/>
       <c r="H442" t="inlineStr"/>
       <c r="I442" t="inlineStr"/>
-      <c r="J442" t="inlineStr"/>
+      <c r="J442" t="inlineStr">
+        <is>
+          <t>Supervision</t>
+        </is>
+      </c>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>01/01/2002</t>
+          <t>01/01/2005</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>02/25/2026</t>
+          <t>12/31/2008</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>Undergraduate and Graduate Admissions Committees</t>
+          <t>Rozita Naghshin (Committee)</t>
         </is>
       </c>
       <c r="D443" t="inlineStr">
         <is>
-          <t>Department of Design and Computation Arts, Concordia University.</t>
+          <t>Software Design as an Aesthetic Design Practice. Concordia University.</t>
         </is>
       </c>
       <c r="E443" t="inlineStr"/>
       <c r="F443" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="G443" t="inlineStr"/>
       <c r="H443" t="inlineStr"/>
       <c r="I443" t="inlineStr"/>
-      <c r="J443" t="inlineStr"/>
+      <c r="J443" t="inlineStr">
+        <is>
+          <t>Supervision</t>
+        </is>
+      </c>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>01/01/2005</t>
+          <t>01/01/2025</t>
         </is>
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>12/31/2008</t>
+          <t>02/25/2026</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t>Faculty Research Advisory Committee</t>
+          <t>Melemaikalani Moniz</t>
         </is>
       </c>
       <c r="D444" t="inlineStr">
         <is>
-          <t>Faculty of Fine Arts, Concordia University.</t>
+          <t>Postdoctoral Fellow in Abundant Soils. Concordia University.</t>
         </is>
       </c>
       <c r="E444" t="inlineStr"/>
       <c r="F444" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Postdoc</t>
         </is>
       </c>
       <c r="G444" t="inlineStr"/>
       <c r="H444" t="inlineStr"/>
       <c r="I444" t="inlineStr"/>
-      <c r="J444" t="inlineStr"/>
+      <c r="J444" t="inlineStr">
+        <is>
+          <t>Supervision</t>
+        </is>
+      </c>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>01/01/2005</t>
+          <t>01/01/2024</t>
         </is>
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>12/31/2008</t>
+          <t>12/31/2026</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t>Hexagram-Concordia Steering Committee</t>
+          <t>Ceyda Yolgörmez</t>
         </is>
       </c>
       <c r="D445" t="inlineStr">
         <is>
-          <t>Concordia University.</t>
+          <t>Horizon Postdoctoral Fellow in Abundant Intelligences. Concordia University.</t>
         </is>
       </c>
       <c r="E445" t="inlineStr"/>
       <c r="F445" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Postdoc</t>
         </is>
       </c>
       <c r="G445" t="inlineStr"/>
       <c r="H445" t="inlineStr"/>
       <c r="I445" t="inlineStr"/>
-      <c r="J445" t="inlineStr"/>
+      <c r="J445" t="inlineStr">
+        <is>
+          <t>Supervision</t>
+        </is>
+      </c>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
         <is>
-          <t>01/01/2020</t>
+          <t>01/01/2019</t>
         </is>
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>02/25/2026</t>
+          <t>12/31/2021</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
         <is>
-          <t>Co-director, Indigenous Futures Research Center</t>
+          <t>Leuli Eschraghi</t>
         </is>
       </c>
       <c r="D446" t="inlineStr">
         <is>
-          <t>Concordia University.</t>
+          <t>Horizon Postdoctoral Fellow in Indigenous Futures. Concordia University.</t>
         </is>
       </c>
       <c r="E446" t="inlineStr"/>
       <c r="F446" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Postdoc</t>
         </is>
       </c>
       <c r="G446" t="inlineStr"/>
       <c r="H446" t="inlineStr"/>
       <c r="I446" t="inlineStr"/>
-      <c r="J446" t="inlineStr"/>
+      <c r="J446" t="inlineStr">
+        <is>
+          <t>Supervision</t>
+        </is>
+      </c>
     </row>
     <row r="447">
       <c r="A447" t="inlineStr">
         <is>
-          <t>01/01/2020</t>
+          <t>01/01/2010</t>
         </is>
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>02/25/2026</t>
+          <t>12/31/2018</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t>Indigenous Directions Leadership Council</t>
+          <t>Acting Chair</t>
         </is>
       </c>
       <c r="D447" t="inlineStr">
         <is>
-          <t>Concordia University.</t>
+          <t>Department of Design and Computation Arts, Concordia University. Various 1-to-2-week terms.</t>
         </is>
       </c>
       <c r="E447" t="inlineStr"/>
@@ -16879,22 +16919,22 @@
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t>01/01/2015</t>
+          <t>09/01/2003</t>
         </is>
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>02/25/2026</t>
+          <t>08/31/2013</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
         <is>
-          <t>Milieux Research Institute Advisory Board</t>
+          <t>Computation Arts Undergraduate Program Director / Co-director</t>
         </is>
       </c>
       <c r="D448" t="inlineStr">
         <is>
-          <t>Concordia University.</t>
+          <t>Department of Design and Computation Arts, Concordia University.</t>
         </is>
       </c>
       <c r="E448" t="inlineStr"/>
@@ -16911,22 +16951,22 @@
     <row r="449">
       <c r="A449" t="inlineStr">
         <is>
-          <t>01/01/2015</t>
+          <t>09/01/2005</t>
         </is>
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>12/31/2018</t>
+          <t>08/31/2008</t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
         <is>
-          <t>Senate Research Committee</t>
+          <t>Graduate Program Director</t>
         </is>
       </c>
       <c r="D449" t="inlineStr">
         <is>
-          <t>Concordia University.</t>
+          <t>Department of Design and Computation Arts, Concordia University.</t>
         </is>
       </c>
       <c r="E449" t="inlineStr"/>
@@ -16943,22 +16983,22 @@
     <row r="450">
       <c r="A450" t="inlineStr">
         <is>
-          <t>01/01/2009</t>
+          <t>09/01/2003</t>
         </is>
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>12/31/2018</t>
+          <t>08/31/2014</t>
         </is>
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t>Board Member (Founding), Research Centre on Technoculture, Art and Gaming (TAG)</t>
+          <t>Computation Lab Director</t>
         </is>
       </c>
       <c r="D450" t="inlineStr">
         <is>
-          <t>Concordia University.</t>
+          <t>Department of Design and Computation Arts, Concordia University.</t>
         </is>
       </c>
       <c r="E450" t="inlineStr"/>
@@ -16975,22 +17015,22 @@
     <row r="451">
       <c r="A451" t="inlineStr">
         <is>
-          <t>01/01/2011</t>
+          <t>01/01/2008</t>
         </is>
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>12/31/2014</t>
+          <t>12/31/2020</t>
         </is>
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t>Faculty Senate</t>
+          <t>Personnel Committee</t>
         </is>
       </c>
       <c r="D451" t="inlineStr">
         <is>
-          <t>Concordia University.</t>
+          <t>Department of Design and Computation Arts, Concordia University.</t>
         </is>
       </c>
       <c r="E451" t="inlineStr"/>
@@ -17007,22 +17047,22 @@
     <row r="452">
       <c r="A452" t="inlineStr">
         <is>
-          <t>01/01/2025</t>
+          <t>01/01/2002</t>
         </is>
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>12/31/2028</t>
+          <t>12/31/2014</t>
         </is>
       </c>
       <c r="C452" t="inlineStr">
         <is>
-          <t>Advisory Board, Digital Technologies Research Centre</t>
+          <t>CART Curriculum Committee, Chair</t>
         </is>
       </c>
       <c r="D452" t="inlineStr">
         <is>
-          <t>National Research Council of Canada.</t>
+          <t>Department of Design and Computation Arts, Concordia University.</t>
         </is>
       </c>
       <c r="E452" t="inlineStr"/>
@@ -17039,22 +17079,22 @@
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t>01/01/2021</t>
+          <t>01/01/2002</t>
         </is>
       </c>
       <c r="B453" t="inlineStr">
         <is>
-          <t>12/31/2023</t>
+          <t>02/25/2026</t>
         </is>
       </c>
       <c r="C453" t="inlineStr">
         <is>
-          <t>Advisory Council on Artificial Intelligence</t>
+          <t>Undergraduate and Graduate Admissions Committees</t>
         </is>
       </c>
       <c r="D453" t="inlineStr">
         <is>
-          <t>Government of Canada.</t>
+          <t>Department of Design and Computation Arts, Concordia University.</t>
         </is>
       </c>
       <c r="E453" t="inlineStr"/>
@@ -17071,20 +17111,24 @@
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t>01/01/2020</t>
+          <t>01/01/2005</t>
         </is>
       </c>
       <c r="B454" t="inlineStr">
         <is>
-          <t>12/31/2022</t>
+          <t>12/31/2008</t>
         </is>
       </c>
       <c r="C454" t="inlineStr">
         <is>
-          <t>Canadian Commission for UNESCO Working Groups on AI Ethics &amp; the Sustainable Development Goals</t>
-        </is>
-      </c>
-      <c r="D454" t="inlineStr"/>
+          <t>Faculty Research Advisory Committee</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>Faculty of Fine Arts, Concordia University.</t>
+        </is>
+      </c>
       <c r="E454" t="inlineStr"/>
       <c r="F454" t="inlineStr">
         <is>
@@ -17099,20 +17143,24 @@
     <row r="455">
       <c r="A455" t="inlineStr">
         <is>
-          <t>01/01/2016</t>
+          <t>01/01/2005</t>
         </is>
       </c>
       <c r="B455" t="inlineStr">
         <is>
-          <t>12/31/2022</t>
+          <t>12/31/2008</t>
         </is>
       </c>
       <c r="C455" t="inlineStr">
         <is>
-          <t>Board Member, imagineNATIVE Film + Media Arts Festival</t>
-        </is>
-      </c>
-      <c r="D455" t="inlineStr"/>
+          <t>Hexagram-Concordia Steering Committee</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>Concordia University.</t>
+        </is>
+      </c>
       <c r="E455" t="inlineStr"/>
       <c r="F455" t="inlineStr">
         <is>
@@ -17127,20 +17175,24 @@
     <row r="456">
       <c r="A456" t="inlineStr">
         <is>
-          <t>01/01/2010</t>
+          <t>01/01/2020</t>
         </is>
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>12/31/2016</t>
+          <t>02/25/2026</t>
         </is>
       </c>
       <c r="C456" t="inlineStr">
         <is>
-          <t>Founding Member, New Media Advisory Board, imagineNATIVE Film + Media Arts Festival</t>
-        </is>
-      </c>
-      <c r="D456" t="inlineStr"/>
+          <t>Co-director, Indigenous Futures Research Center</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>Concordia University.</t>
+        </is>
+      </c>
       <c r="E456" t="inlineStr"/>
       <c r="F456" t="inlineStr">
         <is>
@@ -17155,7 +17207,7 @@
     <row r="457">
       <c r="A457" t="inlineStr">
         <is>
-          <t>01/01/2006</t>
+          <t>01/01/2020</t>
         </is>
       </c>
       <c r="B457" t="inlineStr">
@@ -17165,10 +17217,14 @@
       </c>
       <c r="C457" t="inlineStr">
         <is>
-          <t>Co-Director, Aboriginal Territories in Cyberspace Research Network</t>
-        </is>
-      </c>
-      <c r="D457" t="inlineStr"/>
+          <t>Indigenous Directions Leadership Council</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>Concordia University.</t>
+        </is>
+      </c>
       <c r="E457" t="inlineStr"/>
       <c r="F457" t="inlineStr">
         <is>
@@ -17183,22 +17239,22 @@
     <row r="458">
       <c r="A458" t="inlineStr">
         <is>
-          <t>01/01/2013</t>
+          <t>01/01/2015</t>
         </is>
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>12/31/2016</t>
+          <t>02/25/2026</t>
         </is>
       </c>
       <c r="C458" t="inlineStr">
         <is>
-          <t>First Peoples Literary Prize Incubating Committee &amp; Founding Advisory Board</t>
+          <t>Milieux Research Institute Advisory Board</t>
         </is>
       </c>
       <c r="D458" t="inlineStr">
         <is>
-          <t>Blue Metropolis International Literary Festival, Montreal, QC.</t>
+          <t>Concordia University.</t>
         </is>
       </c>
       <c r="E458" t="inlineStr"/>
@@ -17212,6 +17268,310 @@
       <c r="I458" t="inlineStr"/>
       <c r="J458" t="inlineStr"/>
     </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>01/01/2015</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>12/31/2018</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>Senate Research Committee</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>Concordia University.</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr"/>
+      <c r="F459" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="G459" t="inlineStr"/>
+      <c r="H459" t="inlineStr"/>
+      <c r="I459" t="inlineStr"/>
+      <c r="J459" t="inlineStr"/>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>01/01/2009</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>12/31/2018</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>Board Member (Founding), Research Centre on Technoculture, Art and Gaming (TAG)</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>Concordia University.</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr"/>
+      <c r="F460" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="G460" t="inlineStr"/>
+      <c r="H460" t="inlineStr"/>
+      <c r="I460" t="inlineStr"/>
+      <c r="J460" t="inlineStr"/>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>01/01/2011</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>12/31/2014</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>Faculty Senate</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>Concordia University.</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr"/>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="G461" t="inlineStr"/>
+      <c r="H461" t="inlineStr"/>
+      <c r="I461" t="inlineStr"/>
+      <c r="J461" t="inlineStr"/>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>01/01/2025</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>12/31/2028</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>Advisory Board, Digital Technologies Research Centre</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>National Research Council of Canada.</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr"/>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="G462" t="inlineStr"/>
+      <c r="H462" t="inlineStr"/>
+      <c r="I462" t="inlineStr"/>
+      <c r="J462" t="inlineStr"/>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>01/01/2021</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>12/31/2023</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>Advisory Council on Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>Government of Canada.</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr"/>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="G463" t="inlineStr"/>
+      <c r="H463" t="inlineStr"/>
+      <c r="I463" t="inlineStr"/>
+      <c r="J463" t="inlineStr"/>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>01/01/2020</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>12/31/2022</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>Canadian Commission for UNESCO Working Groups on AI Ethics &amp; the Sustainable Development Goals</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr"/>
+      <c r="E464" t="inlineStr"/>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="G464" t="inlineStr"/>
+      <c r="H464" t="inlineStr"/>
+      <c r="I464" t="inlineStr"/>
+      <c r="J464" t="inlineStr"/>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>01/01/2016</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>12/31/2022</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>Board Member, imagineNATIVE Film + Media Arts Festival</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr"/>
+      <c r="E465" t="inlineStr"/>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="G465" t="inlineStr"/>
+      <c r="H465" t="inlineStr"/>
+      <c r="I465" t="inlineStr"/>
+      <c r="J465" t="inlineStr"/>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>01/01/2010</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>12/31/2016</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>Founding Member, New Media Advisory Board, imagineNATIVE Film + Media Arts Festival</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr"/>
+      <c r="E466" t="inlineStr"/>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="G466" t="inlineStr"/>
+      <c r="H466" t="inlineStr"/>
+      <c r="I466" t="inlineStr"/>
+      <c r="J466" t="inlineStr"/>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>01/01/2006</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>02/25/2026</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>Co-Director, Aboriginal Territories in Cyberspace Research Network</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr"/>
+      <c r="E467" t="inlineStr"/>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="G467" t="inlineStr"/>
+      <c r="H467" t="inlineStr"/>
+      <c r="I467" t="inlineStr"/>
+      <c r="J467" t="inlineStr"/>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>01/01/2013</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>12/31/2016</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>First Peoples Literary Prize Incubating Committee &amp; Founding Advisory Board</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>Blue Metropolis International Literary Festival, Montreal, QC.</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr"/>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="G468" t="inlineStr"/>
+      <c r="H468" t="inlineStr"/>
+      <c r="I468" t="inlineStr"/>
+      <c r="J468" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Supervision band order: Postdoc → PhD → Masters → Grad Certificate → Undergraduate
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/cv-data/cv.xlsx
+++ b/data/cv-data/cv.xlsx
@@ -15447,7 +15447,7 @@
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>01/01/2024</t>
+          <t>01/01/2025</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
@@ -15457,18 +15457,18 @@
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>Destiny Chescappio</t>
+          <t>Melemaikalani Moniz</t>
         </is>
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Postdoctoral Fellow in Abundant Soils. Concordia University.</t>
         </is>
       </c>
       <c r="E407" t="inlineStr"/>
       <c r="F407" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Postdoc</t>
         </is>
       </c>
       <c r="G407" t="inlineStr"/>
@@ -15488,23 +15488,23 @@
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>02/25/2026</t>
+          <t>12/31/2026</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>Hazel Dreslinski</t>
+          <t>Ceyda Yolgörmez</t>
         </is>
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Horizon Postdoctoral Fellow in Abundant Intelligences. Concordia University.</t>
         </is>
       </c>
       <c r="E408" t="inlineStr"/>
       <c r="F408" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Postdoc</t>
         </is>
       </c>
       <c r="G408" t="inlineStr"/>
@@ -15519,28 +15519,28 @@
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>01/01/2024</t>
+          <t>01/01/2019</t>
         </is>
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>02/25/2026</t>
+          <t>12/31/2021</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>Margaret Summers</t>
+          <t>Leuli Eschraghi</t>
         </is>
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Horizon Postdoctoral Fellow in Indigenous Futures. Concordia University.</t>
         </is>
       </c>
       <c r="E409" t="inlineStr"/>
       <c r="F409" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Postdoc</t>
         </is>
       </c>
       <c r="G409" t="inlineStr"/>
@@ -15555,7 +15555,7 @@
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>01/01/2024</t>
+          <t>01/01/2023</t>
         </is>
       </c>
       <c r="B410" t="inlineStr">
@@ -15565,18 +15565,18 @@
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>Milo Puge</t>
+          <t>Juliet Mackie</t>
         </is>
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Reconstituting Indigenous Identities through Portraiture and Storytelling. Concordia University.</t>
         </is>
       </c>
       <c r="E410" t="inlineStr"/>
       <c r="F410" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="G410" t="inlineStr"/>
@@ -15591,28 +15591,28 @@
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>01/01/2024</t>
+          <t>01/01/2021</t>
         </is>
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>12/31/2025</t>
+          <t>12/31/2024</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>Jerwin Cabaneros</t>
+          <t>Mel Lefebvre</t>
         </is>
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Healing Through Ancestral Skin Marking: Traditional Tattooing as Healing and (Re)connection for Indigenous People. Concordia University.</t>
         </is>
       </c>
       <c r="E411" t="inlineStr"/>
       <c r="F411" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="G411" t="inlineStr"/>
@@ -15627,28 +15627,28 @@
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>01/01/2023</t>
+          <t>01/01/2019</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>02/25/2026</t>
+          <t>12/31/2023</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>Taylor McArthur</t>
+          <t>Jessica Barudin (Co-supervisor)</t>
         </is>
       </c>
       <c r="D412" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Re-connecting Through Women's Teachings, Language and Movement. Concordia University.</t>
         </is>
       </c>
       <c r="E412" t="inlineStr"/>
       <c r="F412" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="G412" t="inlineStr"/>
@@ -15663,28 +15663,28 @@
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>01/01/2023</t>
+          <t>01/01/2017</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>12/31/2024</t>
+          <t>12/31/2023</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>Sarah Hontoy-Major</t>
+          <t>Suzanne Kite</t>
         </is>
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Lakota Epistemology, Performance Practice, and Digital Technology. Concordia University.</t>
         </is>
       </c>
       <c r="E413" t="inlineStr"/>
       <c r="F413" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="G413" t="inlineStr"/>
@@ -15699,28 +15699,28 @@
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>01/01/2023</t>
+          <t>01/01/2017</t>
         </is>
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>12/31/2024</t>
+          <t>02/25/2026</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>Neko Wong-Houle</t>
+          <t>Nafisa Sarwath (Secondary)</t>
         </is>
       </c>
       <c r="D414" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Indigenous knowledge, resilience and adaptive capacity. Concordia University.</t>
         </is>
       </c>
       <c r="E414" t="inlineStr"/>
       <c r="F414" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="G414" t="inlineStr"/>
@@ -15735,28 +15735,28 @@
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>01/01/2023</t>
+          <t>01/01/2016</t>
         </is>
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>12/31/2024</t>
+          <t>12/31/2021</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>Ixel Janine</t>
+          <t>Michelle Brown (Secondary)</t>
         </is>
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>(Re)Coding Resurgence: Indigenous Digital Media Kinnections. University of Hawaii Mānoa.</t>
         </is>
       </c>
       <c r="E415" t="inlineStr"/>
       <c r="F415" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="G415" t="inlineStr"/>
@@ -15771,28 +15771,28 @@
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>01/01/2023</t>
+          <t>01/01/2007</t>
         </is>
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>12/31/2023</t>
+          <t>12/31/2014</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>Wan Hua (Wawa) Li</t>
+          <t>Elizabeth LaPensée (Co-supervisor)</t>
         </is>
       </c>
       <c r="D416" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Experiencing Stories: Narrative and Experience in Interactive Media. Simon Fraser University.</t>
         </is>
       </c>
       <c r="E416" t="inlineStr"/>
       <c r="F416" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="G416" t="inlineStr"/>
@@ -15807,28 +15807,28 @@
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>01/01/2023</t>
+          <t>01/01/2008</t>
         </is>
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>12/31/2023</t>
+          <t>12/31/2012</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>Bronson Jacque</t>
+          <t>Miao Song (Secondary)</t>
         </is>
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Experiencing Stories: Narrative and Experience in Interactive Media. Concordia University.</t>
         </is>
       </c>
       <c r="E417" t="inlineStr"/>
       <c r="F417" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="G417" t="inlineStr"/>
@@ -15843,28 +15843,28 @@
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>01/01/2020</t>
+          <t>01/01/2008</t>
         </is>
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>12/31/2024</t>
+          <t>12/31/2011</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>Shirley Ceravolo</t>
+          <t>David Johnston (Secondary)</t>
         </is>
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Aesthetic Animism: Digital Poetry as Ontological Probe. Concordia University.</t>
         </is>
       </c>
       <c r="E418" t="inlineStr"/>
       <c r="F418" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="G418" t="inlineStr"/>
@@ -15879,28 +15879,28 @@
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>01/01/2020</t>
+          <t>01/01/2005</t>
         </is>
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>12/31/2022</t>
+          <t>12/31/2008</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>Alanna Mitchell</t>
+          <t>Rozita Naghshin (Committee)</t>
         </is>
       </c>
       <c r="D419" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Software Design as an Aesthetic Design Practice. Concordia University.</t>
         </is>
       </c>
       <c r="E419" t="inlineStr"/>
       <c r="F419" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="G419" t="inlineStr"/>
@@ -15915,28 +15915,28 @@
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>01/01/2020</t>
+          <t>01/01/2022</t>
         </is>
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>12/31/2021</t>
+          <t>02/25/2026</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>Anthony Lum</t>
+          <t>Vanessa Racine</t>
         </is>
       </c>
       <c r="D420" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Anishinaabe Love: Epistemologies &amp; Videogames. Concordia University.</t>
         </is>
       </c>
       <c r="E420" t="inlineStr"/>
       <c r="F420" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="G420" t="inlineStr"/>
@@ -15951,28 +15951,28 @@
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>01/01/2019</t>
+          <t>01/01/2022</t>
         </is>
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>12/31/2022</t>
+          <t>12/31/2025</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>Unna Regino</t>
+          <t>Tarcisio Cataldi Tegani (Committee)</t>
         </is>
       </c>
       <c r="D421" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Speculative Vexillology: Exploring National Identity and Imagining Afro-Brazilian Futures through Flags. Concordia University.</t>
         </is>
       </c>
       <c r="E421" t="inlineStr"/>
       <c r="F421" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="G421" t="inlineStr"/>
@@ -15987,28 +15987,28 @@
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>01/01/2018</t>
+          <t>01/01/2021</t>
         </is>
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>12/31/2019</t>
+          <t>12/31/2024</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>Alaina Perez</t>
+          <t>Caeleigh Lightning Long</t>
         </is>
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Wawêsiwîn: The Act of Dressing Up — A Research Cree-ation Project. Concordia University.</t>
         </is>
       </c>
       <c r="E422" t="inlineStr"/>
       <c r="F422" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="G422" t="inlineStr"/>
@@ -16023,28 +16023,28 @@
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>01/01/2017</t>
+          <t>01/01/2018</t>
         </is>
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>12/31/2020</t>
+          <t>12/31/2023</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>Kahentawaks Tiewishaw</t>
+          <t>Sébastien Aubin</t>
         </is>
       </c>
       <c r="D423" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Designing Culturally Grounded Cree Syllabaries. Concordia University.</t>
         </is>
       </c>
       <c r="E423" t="inlineStr"/>
       <c r="F423" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="G423" t="inlineStr"/>
@@ -16059,28 +16059,28 @@
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>01/01/2017</t>
+          <t>01/01/2018</t>
         </is>
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>12/31/2019</t>
+          <t>12/31/2021</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>Lucas LaRochelle</t>
+          <t>Waylon Wilson</t>
         </is>
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Tuscarora Virtual Realities. Concordia University.</t>
         </is>
       </c>
       <c r="E424" t="inlineStr"/>
       <c r="F424" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="G424" t="inlineStr"/>
@@ -16105,18 +16105,18 @@
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>Samuelle Bourgault</t>
+          <t>Maize Longboat</t>
         </is>
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Haudenosaunee Storytelling via Video Games. Concordia University.</t>
         </is>
       </c>
       <c r="E425" t="inlineStr"/>
       <c r="F425" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="G425" t="inlineStr"/>
@@ -16131,28 +16131,28 @@
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>01/01/2017</t>
+          <t>01/01/2016</t>
         </is>
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>12/31/2018</t>
+          <t>12/31/2020</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>Alexandria Alcancia-Shaw</t>
+          <t>Nicholas Gwyn Shulman (Co-supervisor)</t>
         </is>
       </c>
       <c r="D426" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Network Arts: Seeing and Making Network Organisms. Concordia University.</t>
         </is>
       </c>
       <c r="E426" t="inlineStr"/>
       <c r="F426" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="G426" t="inlineStr"/>
@@ -16167,28 +16167,28 @@
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>01/01/2017</t>
+          <t>01/01/2014</t>
         </is>
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>12/31/2018</t>
+          <t>12/31/2024</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>Asa Perlman</t>
+          <t>Morgan Kennedy</t>
         </is>
       </c>
       <c r="D427" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Storied Indigeneity in Videogames: Post-Indian Warriors and Indie Japan. Concordia University.</t>
         </is>
       </c>
       <c r="E427" t="inlineStr"/>
       <c r="F427" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="G427" t="inlineStr"/>
@@ -16203,28 +16203,28 @@
     <row r="428">
       <c r="A428" t="inlineStr">
         <is>
-          <t>01/01/2017</t>
+          <t>01/01/2012</t>
         </is>
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>12/31/2018</t>
+          <t>12/31/2015</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>Dion Smith-Dokkie</t>
+          <t>Nikolaos Chandolias (Co-supervisor)</t>
         </is>
       </c>
       <c r="D428" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>KinectEcho: Gesture and Vocal Recognition in New Media, Interactive Art and Live Events. Concordia University.</t>
         </is>
       </c>
       <c r="E428" t="inlineStr"/>
       <c r="F428" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="G428" t="inlineStr"/>
@@ -16239,28 +16239,28 @@
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>01/01/2017</t>
+          <t>01/01/2006</t>
         </is>
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>12/31/2018</t>
+          <t>12/31/2007</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>Eileen Peng</t>
+          <t>Leslie Plumb</t>
         </is>
       </c>
       <c r="D429" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Transversal Entanglements: Research-Creation and the Design Process for Inflexions. Concordia University.</t>
         </is>
       </c>
       <c r="E429" t="inlineStr"/>
       <c r="F429" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="G429" t="inlineStr"/>
@@ -16275,28 +16275,28 @@
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>01/01/2017</t>
+          <t>01/01/2004</t>
         </is>
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>12/31/2018</t>
+          <t>12/31/2008</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>Rudi Aker</t>
+          <t>Mia Song (Co-supervisor)</t>
         </is>
       </c>
       <c r="D430" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Computer-Assisted Interactive Documentary and Performance Arts in Illimitable Space. Concordia University.</t>
         </is>
       </c>
       <c r="E430" t="inlineStr"/>
       <c r="F430" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="G430" t="inlineStr"/>
@@ -16311,28 +16311,28 @@
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>01/01/2017</t>
+          <t>01/01/2003</t>
         </is>
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>12/31/2018</t>
+          <t>12/31/2005</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>Sarah Lauzon</t>
+          <t>Rozita Naghshin (Committee)</t>
         </is>
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>CASE Tool Simplification Via Task-Sensitive Metaphor. Concordia University.</t>
         </is>
       </c>
       <c r="E431" t="inlineStr"/>
       <c r="F431" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="G431" t="inlineStr"/>
@@ -16347,28 +16347,28 @@
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>01/01/2017</t>
+          <t>01/01/2014</t>
         </is>
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>12/31/2018</t>
+          <t>12/31/2015</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>Simon-Albert Boudreault</t>
+          <t>Adriana Navarro Sainz</t>
         </is>
       </c>
       <c r="D432" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Concordia University.</t>
         </is>
       </c>
       <c r="E432" t="inlineStr"/>
       <c r="F432" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Grad Certificate</t>
         </is>
       </c>
       <c r="G432" t="inlineStr"/>
@@ -16383,28 +16383,28 @@
     <row r="433">
       <c r="A433" t="inlineStr">
         <is>
-          <t>01/01/2017</t>
+          <t>01/01/2014</t>
         </is>
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>12/31/2018</t>
+          <t>12/31/2015</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t>Victor Ivanov</t>
+          <t>Guillaume Bourdon</t>
         </is>
       </c>
       <c r="D433" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Concordia University.</t>
         </is>
       </c>
       <c r="E433" t="inlineStr"/>
       <c r="F433" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Grad Certificate</t>
         </is>
       </c>
       <c r="G433" t="inlineStr"/>
@@ -16419,28 +16419,28 @@
     <row r="434">
       <c r="A434" t="inlineStr">
         <is>
-          <t>01/01/2016</t>
+          <t>01/01/2012</t>
         </is>
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>12/31/2020</t>
+          <t>12/31/2013</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t>Emmanuelle Forgues</t>
+          <t>Joanna Pederson</t>
         </is>
       </c>
       <c r="D434" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Augmented Reality: Save the Ghost Signs. Concordia University.</t>
         </is>
       </c>
       <c r="E434" t="inlineStr"/>
       <c r="F434" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Grad Certificate</t>
         </is>
       </c>
       <c r="G434" t="inlineStr"/>
@@ -16455,28 +16455,28 @@
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>01/01/2016</t>
+          <t>01/01/2010</t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>12/31/2018</t>
+          <t>12/31/2011</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>Roxanne Sirois</t>
+          <t>Phil Lichti</t>
         </is>
       </c>
       <c r="D435" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>The Soundwalk as Documentary Practice. Concordia University.</t>
         </is>
       </c>
       <c r="E435" t="inlineStr"/>
       <c r="F435" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Grad Certificate</t>
         </is>
       </c>
       <c r="G435" t="inlineStr"/>
@@ -16491,28 +16491,28 @@
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>01/01/2016</t>
+          <t>01/01/2010</t>
         </is>
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>12/31/2018</t>
+          <t>12/31/2011</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>Darian Jacobs</t>
+          <t>Santiago Salciado</t>
         </is>
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Improving the Design Process for Textbooks. Concordia University.</t>
         </is>
       </c>
       <c r="E436" t="inlineStr"/>
       <c r="F436" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Grad Certificate</t>
         </is>
       </c>
       <c r="G436" t="inlineStr"/>
@@ -16527,28 +16527,28 @@
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>01/01/2015</t>
+          <t>01/01/2006</t>
         </is>
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>12/31/2019</t>
+          <t>12/31/2007</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>Travis Mercredi</t>
+          <t>Oliver Tsuji</t>
         </is>
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Narrative in Digital Media. Concordia University.</t>
         </is>
       </c>
       <c r="E437" t="inlineStr"/>
       <c r="F437" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Grad Certificate</t>
         </is>
       </c>
       <c r="G437" t="inlineStr"/>
@@ -16563,28 +16563,28 @@
     <row r="438">
       <c r="A438" t="inlineStr">
         <is>
-          <t>01/01/2015</t>
+          <t>01/01/2005</t>
         </is>
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>12/31/2016</t>
+          <t>12/31/2006</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>David Clark</t>
+          <t>Louis Goupille</t>
         </is>
       </c>
       <c r="D438" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Painterly Approaches to Virtual Environments. Concordia University.</t>
         </is>
       </c>
       <c r="E438" t="inlineStr"/>
       <c r="F438" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Grad Certificate</t>
         </is>
       </c>
       <c r="G438" t="inlineStr"/>
@@ -16599,28 +16599,28 @@
     <row r="439">
       <c r="A439" t="inlineStr">
         <is>
-          <t>01/01/2015</t>
+          <t>01/01/2005</t>
         </is>
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>12/31/2016</t>
+          <t>12/31/2006</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>Christina Biron</t>
+          <t>Thibaut Duverneix</t>
         </is>
       </c>
       <c r="D439" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Concordia University.</t>
         </is>
       </c>
       <c r="E439" t="inlineStr"/>
       <c r="F439" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Grad Certificate</t>
         </is>
       </c>
       <c r="G439" t="inlineStr"/>
@@ -16635,28 +16635,28 @@
     <row r="440">
       <c r="A440" t="inlineStr">
         <is>
-          <t>01/01/2015</t>
+          <t>01/01/2003</t>
         </is>
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>12/31/2016</t>
+          <t>12/31/2004</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
         <is>
-          <t>Nicole Linn</t>
+          <t>Farah Jamaluddin</t>
         </is>
       </c>
       <c r="D440" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Concordia University.</t>
         </is>
       </c>
       <c r="E440" t="inlineStr"/>
       <c r="F440" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Grad Certificate</t>
         </is>
       </c>
       <c r="G440" t="inlineStr"/>
@@ -16671,28 +16671,28 @@
     <row r="441">
       <c r="A441" t="inlineStr">
         <is>
-          <t>01/01/2015</t>
+          <t>01/01/2003</t>
         </is>
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>12/31/2016</t>
+          <t>12/31/2005</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t>Mi Lin Li</t>
+          <t>Dalia Radwan</t>
         </is>
       </c>
       <c r="D441" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Concordia University.</t>
         </is>
       </c>
       <c r="E441" t="inlineStr"/>
       <c r="F441" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Grad Certificate</t>
         </is>
       </c>
       <c r="G441" t="inlineStr"/>
@@ -16707,28 +16707,28 @@
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>01/01/2014</t>
+          <t>01/01/2002</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>12/31/2018</t>
+          <t>12/31/2003</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>Lianne Maritzer</t>
+          <t>John Stuart</t>
         </is>
       </c>
       <c r="D442" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Concordia University.</t>
         </is>
       </c>
       <c r="E442" t="inlineStr"/>
       <c r="F442" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Grad Certificate</t>
         </is>
       </c>
       <c r="G442" t="inlineStr"/>
@@ -16743,28 +16743,28 @@
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>01/01/2014</t>
+          <t>01/01/2002</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>12/31/2018</t>
+          <t>12/31/2003</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>Julian Glass-Pilon</t>
+          <t>Justyna Latek</t>
         </is>
       </c>
       <c r="D443" t="inlineStr">
         <is>
-          <t>Undergraduate Research Assistant. Concordia University.</t>
+          <t>Concordia University.</t>
         </is>
       </c>
       <c r="E443" t="inlineStr"/>
       <c r="F443" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Grad Certificate</t>
         </is>
       </c>
       <c r="G443" t="inlineStr"/>
@@ -16779,17 +16779,17 @@
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>01/01/2014</t>
+          <t>01/01/2024</t>
         </is>
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>12/31/2016</t>
+          <t>02/25/2026</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t>Erica Perrault</t>
+          <t>Destiny Chescappio</t>
         </is>
       </c>
       <c r="D444" t="inlineStr">
@@ -16815,17 +16815,17 @@
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>01/01/2014</t>
+          <t>01/01/2024</t>
         </is>
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>12/31/2016</t>
+          <t>02/25/2026</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t>Charles Hannah</t>
+          <t>Hazel Dreslinski</t>
         </is>
       </c>
       <c r="D445" t="inlineStr">
@@ -16851,17 +16851,17 @@
     <row r="446">
       <c r="A446" t="inlineStr">
         <is>
-          <t>01/01/2014</t>
+          <t>01/01/2024</t>
         </is>
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>12/31/2015</t>
+          <t>02/25/2026</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
         <is>
-          <t>Nather Aylomen</t>
+          <t>Margaret Summers</t>
         </is>
       </c>
       <c r="D446" t="inlineStr">
@@ -16887,17 +16887,17 @@
     <row r="447">
       <c r="A447" t="inlineStr">
         <is>
-          <t>01/01/2013</t>
+          <t>01/01/2024</t>
         </is>
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>12/31/2015</t>
+          <t>02/25/2026</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t>Näiade Aoun</t>
+          <t>Milo Puge</t>
         </is>
       </c>
       <c r="D447" t="inlineStr">
@@ -16923,17 +16923,17 @@
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t>01/01/2013</t>
+          <t>01/01/2024</t>
         </is>
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>12/31/2015</t>
+          <t>12/31/2025</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
         <is>
-          <t>Alicia McDonald-Fortier</t>
+          <t>Jerwin Cabaneros</t>
         </is>
       </c>
       <c r="D448" t="inlineStr">
@@ -16959,17 +16959,17 @@
     <row r="449">
       <c r="A449" t="inlineStr">
         <is>
-          <t>01/01/2013</t>
+          <t>01/01/2023</t>
         </is>
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>12/31/2015</t>
+          <t>02/25/2026</t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
         <is>
-          <t>Serge Maheau</t>
+          <t>Taylor McArthur</t>
         </is>
       </c>
       <c r="D449" t="inlineStr">
@@ -16995,17 +16995,17 @@
     <row r="450">
       <c r="A450" t="inlineStr">
         <is>
-          <t>01/01/2012</t>
+          <t>01/01/2023</t>
         </is>
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>12/31/2014</t>
+          <t>12/31/2024</t>
         </is>
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t>David Mongeau-Petitepas</t>
+          <t>Sarah Hontoy-Major</t>
         </is>
       </c>
       <c r="D450" t="inlineStr">
@@ -17031,17 +17031,17 @@
     <row r="451">
       <c r="A451" t="inlineStr">
         <is>
-          <t>01/01/2012</t>
+          <t>01/01/2023</t>
         </is>
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>12/31/2014</t>
+          <t>12/31/2024</t>
         </is>
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t>Saurabh Oberoi</t>
+          <t>Neko Wong-Houle</t>
         </is>
       </c>
       <c r="D451" t="inlineStr">
@@ -17067,17 +17067,17 @@
     <row r="452">
       <c r="A452" t="inlineStr">
         <is>
-          <t>01/01/2012</t>
+          <t>01/01/2023</t>
         </is>
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>12/31/2013</t>
+          <t>12/31/2024</t>
         </is>
       </c>
       <c r="C452" t="inlineStr">
         <is>
-          <t>Andy Lunga</t>
+          <t>Ixel Janine</t>
         </is>
       </c>
       <c r="D452" t="inlineStr">
@@ -17103,17 +17103,17 @@
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t>01/01/2012</t>
+          <t>01/01/2023</t>
         </is>
       </c>
       <c r="B453" t="inlineStr">
         <is>
-          <t>12/31/2012</t>
+          <t>12/31/2023</t>
         </is>
       </c>
       <c r="C453" t="inlineStr">
         <is>
-          <t>Bronson Zgeb</t>
+          <t>Wan Hua (Wawa) Li</t>
         </is>
       </c>
       <c r="D453" t="inlineStr">
@@ -17139,17 +17139,17 @@
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t>01/01/2011</t>
+          <t>01/01/2023</t>
         </is>
       </c>
       <c r="B454" t="inlineStr">
         <is>
-          <t>12/31/2012</t>
+          <t>12/31/2023</t>
         </is>
       </c>
       <c r="C454" t="inlineStr">
         <is>
-          <t>Megan Whyte</t>
+          <t>Bronson Jacque</t>
         </is>
       </c>
       <c r="D454" t="inlineStr">
@@ -17175,17 +17175,17 @@
     <row r="455">
       <c r="A455" t="inlineStr">
         <is>
-          <t>01/01/2011</t>
+          <t>01/01/2020</t>
         </is>
       </c>
       <c r="B455" t="inlineStr">
         <is>
-          <t>12/31/2011</t>
+          <t>12/31/2024</t>
         </is>
       </c>
       <c r="C455" t="inlineStr">
         <is>
-          <t>Laura Sirois</t>
+          <t>Shirley Ceravolo</t>
         </is>
       </c>
       <c r="D455" t="inlineStr">
@@ -17211,17 +17211,17 @@
     <row r="456">
       <c r="A456" t="inlineStr">
         <is>
-          <t>01/01/2011</t>
+          <t>01/01/2020</t>
         </is>
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>12/31/2011</t>
+          <t>12/31/2022</t>
         </is>
       </c>
       <c r="C456" t="inlineStr">
         <is>
-          <t>Robert Brais</t>
+          <t>Alanna Mitchell</t>
         </is>
       </c>
       <c r="D456" t="inlineStr">
@@ -17247,17 +17247,17 @@
     <row r="457">
       <c r="A457" t="inlineStr">
         <is>
-          <t>01/01/2011</t>
+          <t>01/01/2020</t>
         </is>
       </c>
       <c r="B457" t="inlineStr">
         <is>
-          <t>12/31/2011</t>
+          <t>12/31/2021</t>
         </is>
       </c>
       <c r="C457" t="inlineStr">
         <is>
-          <t>Marie-Joelle Gringas</t>
+          <t>Anthony Lum</t>
         </is>
       </c>
       <c r="D457" t="inlineStr">
@@ -17283,17 +17283,17 @@
     <row r="458">
       <c r="A458" t="inlineStr">
         <is>
-          <t>01/01/2011</t>
+          <t>01/01/2019</t>
         </is>
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>12/31/2011</t>
+          <t>12/31/2022</t>
         </is>
       </c>
       <c r="C458" t="inlineStr">
         <is>
-          <t>Natalie Pan</t>
+          <t>Unna Regino</t>
         </is>
       </c>
       <c r="D458" t="inlineStr">
@@ -17319,17 +17319,17 @@
     <row r="459">
       <c r="A459" t="inlineStr">
         <is>
-          <t>01/01/2010</t>
+          <t>01/01/2018</t>
         </is>
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>12/31/2015</t>
+          <t>12/31/2019</t>
         </is>
       </c>
       <c r="C459" t="inlineStr">
         <is>
-          <t>Chris Drogaris</t>
+          <t>Alaina Perez</t>
         </is>
       </c>
       <c r="D459" t="inlineStr">
@@ -17355,17 +17355,17 @@
     <row r="460">
       <c r="A460" t="inlineStr">
         <is>
-          <t>01/01/2010</t>
+          <t>01/01/2017</t>
         </is>
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>12/31/2011</t>
+          <t>12/31/2020</t>
         </is>
       </c>
       <c r="C460" t="inlineStr">
         <is>
-          <t>Tania Alvarez</t>
+          <t>Kahentawaks Tiewishaw</t>
         </is>
       </c>
       <c r="D460" t="inlineStr">
@@ -17391,17 +17391,17 @@
     <row r="461">
       <c r="A461" t="inlineStr">
         <is>
-          <t>01/01/2010</t>
+          <t>01/01/2017</t>
         </is>
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>12/31/2010</t>
+          <t>12/31/2019</t>
         </is>
       </c>
       <c r="C461" t="inlineStr">
         <is>
-          <t>Chris Gratton</t>
+          <t>Lucas LaRochelle</t>
         </is>
       </c>
       <c r="D461" t="inlineStr">
@@ -17427,17 +17427,17 @@
     <row r="462">
       <c r="A462" t="inlineStr">
         <is>
-          <t>01/01/2010</t>
+          <t>01/01/2017</t>
         </is>
       </c>
       <c r="B462" t="inlineStr">
         <is>
-          <t>12/31/2010</t>
+          <t>12/31/2019</t>
         </is>
       </c>
       <c r="C462" t="inlineStr">
         <is>
-          <t>Brian Li</t>
+          <t>Samuelle Bourgault</t>
         </is>
       </c>
       <c r="D462" t="inlineStr">
@@ -17463,17 +17463,17 @@
     <row r="463">
       <c r="A463" t="inlineStr">
         <is>
-          <t>01/01/2010</t>
+          <t>01/01/2017</t>
         </is>
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>12/31/2010</t>
+          <t>12/31/2018</t>
         </is>
       </c>
       <c r="C463" t="inlineStr">
         <is>
-          <t>Charles-Antoine Dupont</t>
+          <t>Alexandria Alcancia-Shaw</t>
         </is>
       </c>
       <c r="D463" t="inlineStr">
@@ -17499,17 +17499,17 @@
     <row r="464">
       <c r="A464" t="inlineStr">
         <is>
-          <t>01/01/2010</t>
+          <t>01/01/2017</t>
         </is>
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t>12/31/2010</t>
+          <t>12/31/2018</t>
         </is>
       </c>
       <c r="C464" t="inlineStr">
         <is>
-          <t>Ramy Daghistani</t>
+          <t>Asa Perlman</t>
         </is>
       </c>
       <c r="D464" t="inlineStr">
@@ -17535,17 +17535,17 @@
     <row r="465">
       <c r="A465" t="inlineStr">
         <is>
-          <t>01/01/2009</t>
+          <t>01/01/2017</t>
         </is>
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>12/31/2013</t>
+          <t>12/31/2018</t>
         </is>
       </c>
       <c r="C465" t="inlineStr">
         <is>
-          <t>Charlotte Fischer</t>
+          <t>Dion Smith-Dokkie</t>
         </is>
       </c>
       <c r="D465" t="inlineStr">
@@ -17571,17 +17571,17 @@
     <row r="466">
       <c r="A466" t="inlineStr">
         <is>
-          <t>01/01/2009</t>
+          <t>01/01/2017</t>
         </is>
       </c>
       <c r="B466" t="inlineStr">
         <is>
-          <t>12/31/2013</t>
+          <t>12/31/2018</t>
         </is>
       </c>
       <c r="C466" t="inlineStr">
         <is>
-          <t>Sahar Homami</t>
+          <t>Eileen Peng</t>
         </is>
       </c>
       <c r="D466" t="inlineStr">
@@ -17607,17 +17607,17 @@
     <row r="467">
       <c r="A467" t="inlineStr">
         <is>
-          <t>01/01/2007</t>
+          <t>01/01/2017</t>
         </is>
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>12/31/2013</t>
+          <t>12/31/2018</t>
         </is>
       </c>
       <c r="C467" t="inlineStr">
         <is>
-          <t>Nancy Elizabeth-Townsend</t>
+          <t>Rudi Aker</t>
         </is>
       </c>
       <c r="D467" t="inlineStr">
@@ -17643,17 +17643,17 @@
     <row r="468">
       <c r="A468" t="inlineStr">
         <is>
-          <t>01/01/2007</t>
+          <t>01/01/2017</t>
         </is>
       </c>
       <c r="B468" t="inlineStr">
         <is>
-          <t>12/31/2011</t>
+          <t>12/31/2018</t>
         </is>
       </c>
       <c r="C468" t="inlineStr">
         <is>
-          <t>Mohannad Al-Khatib</t>
+          <t>Sarah Lauzon</t>
         </is>
       </c>
       <c r="D468" t="inlineStr">
@@ -17679,17 +17679,17 @@
     <row r="469">
       <c r="A469" t="inlineStr">
         <is>
-          <t>01/01/2007</t>
+          <t>01/01/2017</t>
         </is>
       </c>
       <c r="B469" t="inlineStr">
         <is>
-          <t>12/31/2009</t>
+          <t>12/31/2018</t>
         </is>
       </c>
       <c r="C469" t="inlineStr">
         <is>
-          <t>Cassandra Lacombe</t>
+          <t>Simon-Albert Boudreault</t>
         </is>
       </c>
       <c r="D469" t="inlineStr">
@@ -17715,17 +17715,17 @@
     <row r="470">
       <c r="A470" t="inlineStr">
         <is>
-          <t>01/01/2007</t>
+          <t>01/01/2017</t>
         </is>
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>12/31/2009</t>
+          <t>12/31/2018</t>
         </is>
       </c>
       <c r="C470" t="inlineStr">
         <is>
-          <t>Raed Mousa</t>
+          <t>Victor Ivanov</t>
         </is>
       </c>
       <c r="D470" t="inlineStr">
@@ -17751,17 +17751,17 @@
     <row r="471">
       <c r="A471" t="inlineStr">
         <is>
-          <t>01/01/2007</t>
+          <t>01/01/2016</t>
         </is>
       </c>
       <c r="B471" t="inlineStr">
         <is>
-          <t>12/31/2009</t>
+          <t>12/31/2020</t>
         </is>
       </c>
       <c r="C471" t="inlineStr">
         <is>
-          <t>Jessica Butler</t>
+          <t>Emmanuelle Forgues</t>
         </is>
       </c>
       <c r="D471" t="inlineStr">
@@ -17787,17 +17787,17 @@
     <row r="472">
       <c r="A472" t="inlineStr">
         <is>
-          <t>01/01/2007</t>
+          <t>01/01/2016</t>
         </is>
       </c>
       <c r="B472" t="inlineStr">
         <is>
-          <t>12/31/2007</t>
+          <t>12/31/2018</t>
         </is>
       </c>
       <c r="C472" t="inlineStr">
         <is>
-          <t>David Johnston</t>
+          <t>Roxanne Sirois</t>
         </is>
       </c>
       <c r="D472" t="inlineStr">
@@ -17823,17 +17823,17 @@
     <row r="473">
       <c r="A473" t="inlineStr">
         <is>
-          <t>01/01/2006</t>
+          <t>01/01/2016</t>
         </is>
       </c>
       <c r="B473" t="inlineStr">
         <is>
-          <t>12/31/2009</t>
+          <t>12/31/2018</t>
         </is>
       </c>
       <c r="C473" t="inlineStr">
         <is>
-          <t>Lucie Belanger</t>
+          <t>Darian Jacobs</t>
         </is>
       </c>
       <c r="D473" t="inlineStr">
@@ -17859,17 +17859,17 @@
     <row r="474">
       <c r="A474" t="inlineStr">
         <is>
-          <t>01/01/2006</t>
+          <t>01/01/2015</t>
         </is>
       </c>
       <c r="B474" t="inlineStr">
         <is>
-          <t>12/31/2009</t>
+          <t>12/31/2019</t>
         </is>
       </c>
       <c r="C474" t="inlineStr">
         <is>
-          <t>Hughes Bruyere</t>
+          <t>Travis Mercredi</t>
         </is>
       </c>
       <c r="D474" t="inlineStr">
@@ -17895,17 +17895,17 @@
     <row r="475">
       <c r="A475" t="inlineStr">
         <is>
-          <t>01/01/2006</t>
+          <t>01/01/2015</t>
         </is>
       </c>
       <c r="B475" t="inlineStr">
         <is>
-          <t>12/31/2009</t>
+          <t>12/31/2016</t>
         </is>
       </c>
       <c r="C475" t="inlineStr">
         <is>
-          <t>Elie Zananiri</t>
+          <t>David Clark</t>
         </is>
       </c>
       <c r="D475" t="inlineStr">
@@ -17931,17 +17931,17 @@
     <row r="476">
       <c r="A476" t="inlineStr">
         <is>
-          <t>01/01/2006</t>
+          <t>01/01/2015</t>
         </is>
       </c>
       <c r="B476" t="inlineStr">
         <is>
-          <t>12/31/2007</t>
+          <t>12/31/2016</t>
         </is>
       </c>
       <c r="C476" t="inlineStr">
         <is>
-          <t>Damir Cheremisov</t>
+          <t>Christina Biron</t>
         </is>
       </c>
       <c r="D476" t="inlineStr">
@@ -17967,17 +17967,17 @@
     <row r="477">
       <c r="A477" t="inlineStr">
         <is>
-          <t>01/01/2006</t>
+          <t>01/01/2015</t>
         </is>
       </c>
       <c r="B477" t="inlineStr">
         <is>
-          <t>12/31/2006</t>
+          <t>12/31/2016</t>
         </is>
       </c>
       <c r="C477" t="inlineStr">
         <is>
-          <t>Thierry Giles</t>
+          <t>Nicole Linn</t>
         </is>
       </c>
       <c r="D477" t="inlineStr">
@@ -18003,17 +18003,17 @@
     <row r="478">
       <c r="A478" t="inlineStr">
         <is>
-          <t>01/01/2006</t>
+          <t>01/01/2015</t>
         </is>
       </c>
       <c r="B478" t="inlineStr">
         <is>
-          <t>12/31/2006</t>
+          <t>12/31/2016</t>
         </is>
       </c>
       <c r="C478" t="inlineStr">
         <is>
-          <t>Lysanne Bellemare</t>
+          <t>Mi Lin Li</t>
         </is>
       </c>
       <c r="D478" t="inlineStr">
@@ -18039,17 +18039,17 @@
     <row r="479">
       <c r="A479" t="inlineStr">
         <is>
-          <t>01/01/2005</t>
+          <t>01/01/2014</t>
         </is>
       </c>
       <c r="B479" t="inlineStr">
         <is>
-          <t>12/31/2008</t>
+          <t>12/31/2018</t>
         </is>
       </c>
       <c r="C479" t="inlineStr">
         <is>
-          <t>Yannick Assogba</t>
+          <t>Lianne Maritzer</t>
         </is>
       </c>
       <c r="D479" t="inlineStr">
@@ -18075,17 +18075,17 @@
     <row r="480">
       <c r="A480" t="inlineStr">
         <is>
-          <t>01/01/2005</t>
+          <t>01/01/2014</t>
         </is>
       </c>
       <c r="B480" t="inlineStr">
         <is>
-          <t>12/31/2008</t>
+          <t>12/31/2018</t>
         </is>
       </c>
       <c r="C480" t="inlineStr">
         <is>
-          <t>Maroussia Lévesque</t>
+          <t>Julian Glass-Pilon</t>
         </is>
       </c>
       <c r="D480" t="inlineStr">
@@ -18111,17 +18111,17 @@
     <row r="481">
       <c r="A481" t="inlineStr">
         <is>
-          <t>01/01/2005</t>
+          <t>01/01/2014</t>
         </is>
       </c>
       <c r="B481" t="inlineStr">
         <is>
-          <t>12/31/2008</t>
+          <t>12/31/2016</t>
         </is>
       </c>
       <c r="C481" t="inlineStr">
         <is>
-          <t>Morgan Kennedy</t>
+          <t>Erica Perrault</t>
         </is>
       </c>
       <c r="D481" t="inlineStr">
@@ -18147,17 +18147,17 @@
     <row r="482">
       <c r="A482" t="inlineStr">
         <is>
-          <t>01/01/2005</t>
+          <t>01/01/2014</t>
         </is>
       </c>
       <c r="B482" t="inlineStr">
         <is>
-          <t>12/31/2005</t>
+          <t>12/31/2016</t>
         </is>
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>Liu Zehuan</t>
+          <t>Charles Hannah</t>
         </is>
       </c>
       <c r="D482" t="inlineStr">
@@ -18183,17 +18183,17 @@
     <row r="483">
       <c r="A483" t="inlineStr">
         <is>
-          <t>01/01/2005</t>
+          <t>01/01/2014</t>
         </is>
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>12/31/2005</t>
+          <t>12/31/2015</t>
         </is>
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>Hoda Adra</t>
+          <t>Nather Aylomen</t>
         </is>
       </c>
       <c r="D483" t="inlineStr">
@@ -18219,17 +18219,17 @@
     <row r="484">
       <c r="A484" t="inlineStr">
         <is>
-          <t>01/01/2005</t>
+          <t>01/01/2013</t>
         </is>
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>12/31/2005</t>
+          <t>12/31/2015</t>
         </is>
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>Elana Rudick</t>
+          <t>Näiade Aoun</t>
         </is>
       </c>
       <c r="D484" t="inlineStr">
@@ -18255,17 +18255,17 @@
     <row r="485">
       <c r="A485" t="inlineStr">
         <is>
-          <t>01/01/2004</t>
+          <t>01/01/2013</t>
         </is>
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>12/31/2004</t>
+          <t>12/31/2015</t>
         </is>
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>Thanh Pham</t>
+          <t>Alicia McDonald-Fortier</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
@@ -18291,17 +18291,17 @@
     <row r="486">
       <c r="A486" t="inlineStr">
         <is>
-          <t>01/01/2004</t>
+          <t>01/01/2013</t>
         </is>
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>12/31/2004</t>
+          <t>12/31/2015</t>
         </is>
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>Elio Bidinost</t>
+          <t>Serge Maheau</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
@@ -18327,17 +18327,17 @@
     <row r="487">
       <c r="A487" t="inlineStr">
         <is>
-          <t>01/01/2003</t>
+          <t>01/01/2012</t>
         </is>
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>12/31/2005</t>
+          <t>12/31/2014</t>
         </is>
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>Bruno Nadeau</t>
+          <t>David Mongeau-Petitepas</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
@@ -18363,17 +18363,17 @@
     <row r="488">
       <c r="A488" t="inlineStr">
         <is>
-          <t>01/01/2003</t>
+          <t>01/01/2012</t>
         </is>
       </c>
       <c r="B488" t="inlineStr">
         <is>
-          <t>12/31/2005</t>
+          <t>12/31/2014</t>
         </is>
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>David Bouchard</t>
+          <t>Saurabh Oberoi</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
@@ -18399,17 +18399,17 @@
     <row r="489">
       <c r="A489" t="inlineStr">
         <is>
-          <t>01/01/2003</t>
+          <t>01/01/2012</t>
         </is>
       </c>
       <c r="B489" t="inlineStr">
         <is>
-          <t>12/31/2005</t>
+          <t>12/31/2013</t>
         </is>
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>Frank Tsonis</t>
+          <t>Andy Lunga</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
@@ -18435,17 +18435,17 @@
     <row r="490">
       <c r="A490" t="inlineStr">
         <is>
-          <t>01/01/2003</t>
+          <t>01/01/2012</t>
         </is>
       </c>
       <c r="B490" t="inlineStr">
         <is>
-          <t>12/31/2003</t>
+          <t>12/31/2012</t>
         </is>
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>Katia Minarikova</t>
+          <t>Bronson Zgeb</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
@@ -18471,17 +18471,17 @@
     <row r="491">
       <c r="A491" t="inlineStr">
         <is>
-          <t>01/01/2003</t>
+          <t>01/01/2011</t>
         </is>
       </c>
       <c r="B491" t="inlineStr">
         <is>
-          <t>12/31/2003</t>
+          <t>12/31/2012</t>
         </is>
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>Jonathan Joseph</t>
+          <t>Megan Whyte</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
@@ -18507,17 +18507,17 @@
     <row r="492">
       <c r="A492" t="inlineStr">
         <is>
-          <t>01/01/2003</t>
+          <t>01/01/2011</t>
         </is>
       </c>
       <c r="B492" t="inlineStr">
         <is>
-          <t>12/31/2003</t>
+          <t>12/31/2011</t>
         </is>
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>David Johnston</t>
+          <t>Laura Sirois</t>
         </is>
       </c>
       <c r="D492" t="inlineStr">
@@ -18543,28 +18543,28 @@
     <row r="493">
       <c r="A493" t="inlineStr">
         <is>
-          <t>01/01/2014</t>
+          <t>01/01/2011</t>
         </is>
       </c>
       <c r="B493" t="inlineStr">
         <is>
-          <t>12/31/2015</t>
+          <t>12/31/2011</t>
         </is>
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>Adriana Navarro Sainz</t>
+          <t>Robert Brais</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
         <is>
-          <t>Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E493" t="inlineStr"/>
       <c r="F493" t="inlineStr">
         <is>
-          <t>Grad Certificate</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G493" t="inlineStr"/>
@@ -18579,28 +18579,28 @@
     <row r="494">
       <c r="A494" t="inlineStr">
         <is>
-          <t>01/01/2014</t>
+          <t>01/01/2011</t>
         </is>
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>12/31/2015</t>
+          <t>12/31/2011</t>
         </is>
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>Guillaume Bourdon</t>
+          <t>Marie-Joelle Gringas</t>
         </is>
       </c>
       <c r="D494" t="inlineStr">
         <is>
-          <t>Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E494" t="inlineStr"/>
       <c r="F494" t="inlineStr">
         <is>
-          <t>Grad Certificate</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G494" t="inlineStr"/>
@@ -18615,28 +18615,28 @@
     <row r="495">
       <c r="A495" t="inlineStr">
         <is>
-          <t>01/01/2012</t>
+          <t>01/01/2011</t>
         </is>
       </c>
       <c r="B495" t="inlineStr">
         <is>
-          <t>12/31/2013</t>
+          <t>12/31/2011</t>
         </is>
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>Joanna Pederson</t>
+          <t>Natalie Pan</t>
         </is>
       </c>
       <c r="D495" t="inlineStr">
         <is>
-          <t>Augmented Reality: Save the Ghost Signs. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E495" t="inlineStr"/>
       <c r="F495" t="inlineStr">
         <is>
-          <t>Grad Certificate</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G495" t="inlineStr"/>
@@ -18656,23 +18656,23 @@
       </c>
       <c r="B496" t="inlineStr">
         <is>
-          <t>12/31/2011</t>
+          <t>12/31/2015</t>
         </is>
       </c>
       <c r="C496" t="inlineStr">
         <is>
-          <t>Phil Lichti</t>
+          <t>Chris Drogaris</t>
         </is>
       </c>
       <c r="D496" t="inlineStr">
         <is>
-          <t>The Soundwalk as Documentary Practice. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E496" t="inlineStr"/>
       <c r="F496" t="inlineStr">
         <is>
-          <t>Grad Certificate</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G496" t="inlineStr"/>
@@ -18697,18 +18697,18 @@
       </c>
       <c r="C497" t="inlineStr">
         <is>
-          <t>Santiago Salciado</t>
+          <t>Tania Alvarez</t>
         </is>
       </c>
       <c r="D497" t="inlineStr">
         <is>
-          <t>Improving the Design Process for Textbooks. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E497" t="inlineStr"/>
       <c r="F497" t="inlineStr">
         <is>
-          <t>Grad Certificate</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G497" t="inlineStr"/>
@@ -18723,28 +18723,28 @@
     <row r="498">
       <c r="A498" t="inlineStr">
         <is>
-          <t>01/01/2006</t>
+          <t>01/01/2010</t>
         </is>
       </c>
       <c r="B498" t="inlineStr">
         <is>
-          <t>12/31/2007</t>
+          <t>12/31/2010</t>
         </is>
       </c>
       <c r="C498" t="inlineStr">
         <is>
-          <t>Oliver Tsuji</t>
+          <t>Chris Gratton</t>
         </is>
       </c>
       <c r="D498" t="inlineStr">
         <is>
-          <t>Narrative in Digital Media. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E498" t="inlineStr"/>
       <c r="F498" t="inlineStr">
         <is>
-          <t>Grad Certificate</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G498" t="inlineStr"/>
@@ -18759,28 +18759,28 @@
     <row r="499">
       <c r="A499" t="inlineStr">
         <is>
-          <t>01/01/2005</t>
+          <t>01/01/2010</t>
         </is>
       </c>
       <c r="B499" t="inlineStr">
         <is>
-          <t>12/31/2006</t>
+          <t>12/31/2010</t>
         </is>
       </c>
       <c r="C499" t="inlineStr">
         <is>
-          <t>Louis Goupille</t>
+          <t>Brian Li</t>
         </is>
       </c>
       <c r="D499" t="inlineStr">
         <is>
-          <t>Painterly Approaches to Virtual Environments. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E499" t="inlineStr"/>
       <c r="F499" t="inlineStr">
         <is>
-          <t>Grad Certificate</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G499" t="inlineStr"/>
@@ -18795,28 +18795,28 @@
     <row r="500">
       <c r="A500" t="inlineStr">
         <is>
-          <t>01/01/2005</t>
+          <t>01/01/2010</t>
         </is>
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>12/31/2006</t>
+          <t>12/31/2010</t>
         </is>
       </c>
       <c r="C500" t="inlineStr">
         <is>
-          <t>Thibaut Duverneix</t>
+          <t>Charles-Antoine Dupont</t>
         </is>
       </c>
       <c r="D500" t="inlineStr">
         <is>
-          <t>Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E500" t="inlineStr"/>
       <c r="F500" t="inlineStr">
         <is>
-          <t>Grad Certificate</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G500" t="inlineStr"/>
@@ -18831,28 +18831,28 @@
     <row r="501">
       <c r="A501" t="inlineStr">
         <is>
-          <t>01/01/2003</t>
+          <t>01/01/2010</t>
         </is>
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>12/31/2004</t>
+          <t>12/31/2010</t>
         </is>
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>Farah Jamaluddin</t>
+          <t>Ramy Daghistani</t>
         </is>
       </c>
       <c r="D501" t="inlineStr">
         <is>
-          <t>Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E501" t="inlineStr"/>
       <c r="F501" t="inlineStr">
         <is>
-          <t>Grad Certificate</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G501" t="inlineStr"/>
@@ -18867,28 +18867,28 @@
     <row r="502">
       <c r="A502" t="inlineStr">
         <is>
-          <t>01/01/2003</t>
+          <t>01/01/2009</t>
         </is>
       </c>
       <c r="B502" t="inlineStr">
         <is>
-          <t>12/31/2005</t>
+          <t>12/31/2013</t>
         </is>
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>Dalia Radwan</t>
+          <t>Charlotte Fischer</t>
         </is>
       </c>
       <c r="D502" t="inlineStr">
         <is>
-          <t>Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E502" t="inlineStr"/>
       <c r="F502" t="inlineStr">
         <is>
-          <t>Grad Certificate</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G502" t="inlineStr"/>
@@ -18903,28 +18903,28 @@
     <row r="503">
       <c r="A503" t="inlineStr">
         <is>
-          <t>01/01/2002</t>
+          <t>01/01/2009</t>
         </is>
       </c>
       <c r="B503" t="inlineStr">
         <is>
-          <t>12/31/2003</t>
+          <t>12/31/2013</t>
         </is>
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>John Stuart</t>
+          <t>Sahar Homami</t>
         </is>
       </c>
       <c r="D503" t="inlineStr">
         <is>
-          <t>Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E503" t="inlineStr"/>
       <c r="F503" t="inlineStr">
         <is>
-          <t>Grad Certificate</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G503" t="inlineStr"/>
@@ -18939,28 +18939,28 @@
     <row r="504">
       <c r="A504" t="inlineStr">
         <is>
-          <t>01/01/2002</t>
+          <t>01/01/2007</t>
         </is>
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>12/31/2003</t>
+          <t>12/31/2013</t>
         </is>
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>Justyna Latek</t>
+          <t>Nancy Elizabeth-Townsend</t>
         </is>
       </c>
       <c r="D504" t="inlineStr">
         <is>
-          <t>Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E504" t="inlineStr"/>
       <c r="F504" t="inlineStr">
         <is>
-          <t>Grad Certificate</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G504" t="inlineStr"/>
@@ -18975,28 +18975,28 @@
     <row r="505">
       <c r="A505" t="inlineStr">
         <is>
-          <t>01/01/2022</t>
+          <t>01/01/2007</t>
         </is>
       </c>
       <c r="B505" t="inlineStr">
         <is>
-          <t>02/25/2026</t>
+          <t>12/31/2011</t>
         </is>
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>Vanessa Racine</t>
+          <t>Mohannad Al-Khatib</t>
         </is>
       </c>
       <c r="D505" t="inlineStr">
         <is>
-          <t>Anishinaabe Love: Epistemologies &amp; Videogames. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E505" t="inlineStr"/>
       <c r="F505" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G505" t="inlineStr"/>
@@ -19011,28 +19011,28 @@
     <row r="506">
       <c r="A506" t="inlineStr">
         <is>
-          <t>01/01/2022</t>
+          <t>01/01/2007</t>
         </is>
       </c>
       <c r="B506" t="inlineStr">
         <is>
-          <t>12/31/2025</t>
+          <t>12/31/2009</t>
         </is>
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>Tarcisio Cataldi Tegani (Committee)</t>
+          <t>Cassandra Lacombe</t>
         </is>
       </c>
       <c r="D506" t="inlineStr">
         <is>
-          <t>Speculative Vexillology: Exploring National Identity and Imagining Afro-Brazilian Futures through Flags. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E506" t="inlineStr"/>
       <c r="F506" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G506" t="inlineStr"/>
@@ -19047,28 +19047,28 @@
     <row r="507">
       <c r="A507" t="inlineStr">
         <is>
-          <t>01/01/2021</t>
+          <t>01/01/2007</t>
         </is>
       </c>
       <c r="B507" t="inlineStr">
         <is>
-          <t>12/31/2024</t>
+          <t>12/31/2009</t>
         </is>
       </c>
       <c r="C507" t="inlineStr">
         <is>
-          <t>Caeleigh Lightning Long</t>
+          <t>Raed Mousa</t>
         </is>
       </c>
       <c r="D507" t="inlineStr">
         <is>
-          <t>Wawêsiwîn: The Act of Dressing Up — A Research Cree-ation Project. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E507" t="inlineStr"/>
       <c r="F507" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G507" t="inlineStr"/>
@@ -19083,28 +19083,28 @@
     <row r="508">
       <c r="A508" t="inlineStr">
         <is>
-          <t>01/01/2018</t>
+          <t>01/01/2007</t>
         </is>
       </c>
       <c r="B508" t="inlineStr">
         <is>
-          <t>12/31/2023</t>
+          <t>12/31/2009</t>
         </is>
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>Sébastien Aubin</t>
+          <t>Jessica Butler</t>
         </is>
       </c>
       <c r="D508" t="inlineStr">
         <is>
-          <t>Designing Culturally Grounded Cree Syllabaries. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E508" t="inlineStr"/>
       <c r="F508" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G508" t="inlineStr"/>
@@ -19119,28 +19119,28 @@
     <row r="509">
       <c r="A509" t="inlineStr">
         <is>
-          <t>01/01/2018</t>
+          <t>01/01/2007</t>
         </is>
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>12/31/2021</t>
+          <t>12/31/2007</t>
         </is>
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>Waylon Wilson</t>
+          <t>David Johnston</t>
         </is>
       </c>
       <c r="D509" t="inlineStr">
         <is>
-          <t>Tuscarora Virtual Realities. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E509" t="inlineStr"/>
       <c r="F509" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G509" t="inlineStr"/>
@@ -19155,28 +19155,28 @@
     <row r="510">
       <c r="A510" t="inlineStr">
         <is>
-          <t>01/01/2017</t>
+          <t>01/01/2006</t>
         </is>
       </c>
       <c r="B510" t="inlineStr">
         <is>
-          <t>12/31/2019</t>
+          <t>12/31/2009</t>
         </is>
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>Maize Longboat</t>
+          <t>Lucie Belanger</t>
         </is>
       </c>
       <c r="D510" t="inlineStr">
         <is>
-          <t>Haudenosaunee Storytelling via Video Games. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E510" t="inlineStr"/>
       <c r="F510" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G510" t="inlineStr"/>
@@ -19191,28 +19191,28 @@
     <row r="511">
       <c r="A511" t="inlineStr">
         <is>
-          <t>01/01/2016</t>
+          <t>01/01/2006</t>
         </is>
       </c>
       <c r="B511" t="inlineStr">
         <is>
-          <t>12/31/2020</t>
+          <t>12/31/2009</t>
         </is>
       </c>
       <c r="C511" t="inlineStr">
         <is>
-          <t>Nicholas Gwyn Shulman (Co-supervisor)</t>
+          <t>Hughes Bruyere</t>
         </is>
       </c>
       <c r="D511" t="inlineStr">
         <is>
-          <t>Network Arts: Seeing and Making Network Organisms. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E511" t="inlineStr"/>
       <c r="F511" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G511" t="inlineStr"/>
@@ -19227,28 +19227,28 @@
     <row r="512">
       <c r="A512" t="inlineStr">
         <is>
-          <t>01/01/2014</t>
+          <t>01/01/2006</t>
         </is>
       </c>
       <c r="B512" t="inlineStr">
         <is>
-          <t>12/31/2024</t>
+          <t>12/31/2009</t>
         </is>
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>Morgan Kennedy</t>
+          <t>Elie Zananiri</t>
         </is>
       </c>
       <c r="D512" t="inlineStr">
         <is>
-          <t>Storied Indigeneity in Videogames: Post-Indian Warriors and Indie Japan. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E512" t="inlineStr"/>
       <c r="F512" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G512" t="inlineStr"/>
@@ -19263,28 +19263,28 @@
     <row r="513">
       <c r="A513" t="inlineStr">
         <is>
-          <t>01/01/2012</t>
+          <t>01/01/2006</t>
         </is>
       </c>
       <c r="B513" t="inlineStr">
         <is>
-          <t>12/31/2015</t>
+          <t>12/31/2007</t>
         </is>
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>Nikolaos Chandolias (Co-supervisor)</t>
+          <t>Damir Cheremisov</t>
         </is>
       </c>
       <c r="D513" t="inlineStr">
         <is>
-          <t>KinectEcho: Gesture and Vocal Recognition in New Media, Interactive Art and Live Events. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E513" t="inlineStr"/>
       <c r="F513" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G513" t="inlineStr"/>
@@ -19304,23 +19304,23 @@
       </c>
       <c r="B514" t="inlineStr">
         <is>
-          <t>12/31/2007</t>
+          <t>12/31/2006</t>
         </is>
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>Leslie Plumb</t>
+          <t>Thierry Giles</t>
         </is>
       </c>
       <c r="D514" t="inlineStr">
         <is>
-          <t>Transversal Entanglements: Research-Creation and the Design Process for Inflexions. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E514" t="inlineStr"/>
       <c r="F514" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G514" t="inlineStr"/>
@@ -19335,28 +19335,28 @@
     <row r="515">
       <c r="A515" t="inlineStr">
         <is>
-          <t>01/01/2004</t>
+          <t>01/01/2006</t>
         </is>
       </c>
       <c r="B515" t="inlineStr">
         <is>
-          <t>12/31/2008</t>
+          <t>12/31/2006</t>
         </is>
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>Mia Song (Co-supervisor)</t>
+          <t>Lysanne Bellemare</t>
         </is>
       </c>
       <c r="D515" t="inlineStr">
         <is>
-          <t>Computer-Assisted Interactive Documentary and Performance Arts in Illimitable Space. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E515" t="inlineStr"/>
       <c r="F515" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G515" t="inlineStr"/>
@@ -19371,28 +19371,28 @@
     <row r="516">
       <c r="A516" t="inlineStr">
         <is>
-          <t>01/01/2003</t>
+          <t>01/01/2005</t>
         </is>
       </c>
       <c r="B516" t="inlineStr">
         <is>
-          <t>12/31/2005</t>
+          <t>12/31/2008</t>
         </is>
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>Rozita Naghshin (Committee)</t>
+          <t>Yannick Assogba</t>
         </is>
       </c>
       <c r="D516" t="inlineStr">
         <is>
-          <t>CASE Tool Simplification Via Task-Sensitive Metaphor. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E516" t="inlineStr"/>
       <c r="F516" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G516" t="inlineStr"/>
@@ -19407,28 +19407,28 @@
     <row r="517">
       <c r="A517" t="inlineStr">
         <is>
-          <t>01/01/2023</t>
+          <t>01/01/2005</t>
         </is>
       </c>
       <c r="B517" t="inlineStr">
         <is>
-          <t>02/25/2026</t>
+          <t>12/31/2008</t>
         </is>
       </c>
       <c r="C517" t="inlineStr">
         <is>
-          <t>Juliet Mackie</t>
+          <t>Maroussia Lévesque</t>
         </is>
       </c>
       <c r="D517" t="inlineStr">
         <is>
-          <t>Reconstituting Indigenous Identities through Portraiture and Storytelling. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E517" t="inlineStr"/>
       <c r="F517" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G517" t="inlineStr"/>
@@ -19443,28 +19443,28 @@
     <row r="518">
       <c r="A518" t="inlineStr">
         <is>
-          <t>01/01/2021</t>
+          <t>01/01/2005</t>
         </is>
       </c>
       <c r="B518" t="inlineStr">
         <is>
-          <t>12/31/2024</t>
+          <t>12/31/2008</t>
         </is>
       </c>
       <c r="C518" t="inlineStr">
         <is>
-          <t>Mel Lefebvre</t>
+          <t>Morgan Kennedy</t>
         </is>
       </c>
       <c r="D518" t="inlineStr">
         <is>
-          <t>Healing Through Ancestral Skin Marking: Traditional Tattooing as Healing and (Re)connection for Indigenous People. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E518" t="inlineStr"/>
       <c r="F518" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G518" t="inlineStr"/>
@@ -19479,28 +19479,28 @@
     <row r="519">
       <c r="A519" t="inlineStr">
         <is>
-          <t>01/01/2019</t>
+          <t>01/01/2005</t>
         </is>
       </c>
       <c r="B519" t="inlineStr">
         <is>
-          <t>12/31/2023</t>
+          <t>12/31/2005</t>
         </is>
       </c>
       <c r="C519" t="inlineStr">
         <is>
-          <t>Jessica Barudin (Co-supervisor)</t>
+          <t>Liu Zehuan</t>
         </is>
       </c>
       <c r="D519" t="inlineStr">
         <is>
-          <t>Re-connecting Through Women's Teachings, Language and Movement. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E519" t="inlineStr"/>
       <c r="F519" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G519" t="inlineStr"/>
@@ -19515,28 +19515,28 @@
     <row r="520">
       <c r="A520" t="inlineStr">
         <is>
-          <t>01/01/2017</t>
+          <t>01/01/2005</t>
         </is>
       </c>
       <c r="B520" t="inlineStr">
         <is>
-          <t>12/31/2023</t>
+          <t>12/31/2005</t>
         </is>
       </c>
       <c r="C520" t="inlineStr">
         <is>
-          <t>Suzanne Kite</t>
+          <t>Hoda Adra</t>
         </is>
       </c>
       <c r="D520" t="inlineStr">
         <is>
-          <t>Lakota Epistemology, Performance Practice, and Digital Technology. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E520" t="inlineStr"/>
       <c r="F520" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G520" t="inlineStr"/>
@@ -19551,28 +19551,28 @@
     <row r="521">
       <c r="A521" t="inlineStr">
         <is>
-          <t>01/01/2017</t>
+          <t>01/01/2005</t>
         </is>
       </c>
       <c r="B521" t="inlineStr">
         <is>
-          <t>02/25/2026</t>
+          <t>12/31/2005</t>
         </is>
       </c>
       <c r="C521" t="inlineStr">
         <is>
-          <t>Nafisa Sarwath (Secondary)</t>
+          <t>Elana Rudick</t>
         </is>
       </c>
       <c r="D521" t="inlineStr">
         <is>
-          <t>Indigenous knowledge, resilience and adaptive capacity. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E521" t="inlineStr"/>
       <c r="F521" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G521" t="inlineStr"/>
@@ -19587,28 +19587,28 @@
     <row r="522">
       <c r="A522" t="inlineStr">
         <is>
-          <t>01/01/2016</t>
+          <t>01/01/2004</t>
         </is>
       </c>
       <c r="B522" t="inlineStr">
         <is>
-          <t>12/31/2021</t>
+          <t>12/31/2004</t>
         </is>
       </c>
       <c r="C522" t="inlineStr">
         <is>
-          <t>Michelle Brown (Secondary)</t>
+          <t>Thanh Pham</t>
         </is>
       </c>
       <c r="D522" t="inlineStr">
         <is>
-          <t>(Re)Coding Resurgence: Indigenous Digital Media Kinnections. University of Hawaii Mānoa.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E522" t="inlineStr"/>
       <c r="F522" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G522" t="inlineStr"/>
@@ -19623,28 +19623,28 @@
     <row r="523">
       <c r="A523" t="inlineStr">
         <is>
-          <t>01/01/2007</t>
+          <t>01/01/2004</t>
         </is>
       </c>
       <c r="B523" t="inlineStr">
         <is>
-          <t>12/31/2014</t>
+          <t>12/31/2004</t>
         </is>
       </c>
       <c r="C523" t="inlineStr">
         <is>
-          <t>Elizabeth LaPensée (Co-supervisor)</t>
+          <t>Elio Bidinost</t>
         </is>
       </c>
       <c r="D523" t="inlineStr">
         <is>
-          <t>Experiencing Stories: Narrative and Experience in Interactive Media. Simon Fraser University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E523" t="inlineStr"/>
       <c r="F523" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G523" t="inlineStr"/>
@@ -19659,28 +19659,28 @@
     <row r="524">
       <c r="A524" t="inlineStr">
         <is>
-          <t>01/01/2008</t>
+          <t>01/01/2003</t>
         </is>
       </c>
       <c r="B524" t="inlineStr">
         <is>
-          <t>12/31/2012</t>
+          <t>12/31/2005</t>
         </is>
       </c>
       <c r="C524" t="inlineStr">
         <is>
-          <t>Miao Song (Secondary)</t>
+          <t>Bruno Nadeau</t>
         </is>
       </c>
       <c r="D524" t="inlineStr">
         <is>
-          <t>Experiencing Stories: Narrative and Experience in Interactive Media. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E524" t="inlineStr"/>
       <c r="F524" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G524" t="inlineStr"/>
@@ -19695,28 +19695,28 @@
     <row r="525">
       <c r="A525" t="inlineStr">
         <is>
-          <t>01/01/2008</t>
+          <t>01/01/2003</t>
         </is>
       </c>
       <c r="B525" t="inlineStr">
         <is>
-          <t>12/31/2011</t>
+          <t>12/31/2005</t>
         </is>
       </c>
       <c r="C525" t="inlineStr">
         <is>
-          <t>David Johnston (Secondary)</t>
+          <t>David Bouchard</t>
         </is>
       </c>
       <c r="D525" t="inlineStr">
         <is>
-          <t>Aesthetic Animism: Digital Poetry as Ontological Probe. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E525" t="inlineStr"/>
       <c r="F525" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G525" t="inlineStr"/>
@@ -19731,28 +19731,28 @@
     <row r="526">
       <c r="A526" t="inlineStr">
         <is>
-          <t>01/01/2005</t>
+          <t>01/01/2003</t>
         </is>
       </c>
       <c r="B526" t="inlineStr">
         <is>
-          <t>12/31/2008</t>
+          <t>12/31/2005</t>
         </is>
       </c>
       <c r="C526" t="inlineStr">
         <is>
-          <t>Rozita Naghshin (Committee)</t>
+          <t>Frank Tsonis</t>
         </is>
       </c>
       <c r="D526" t="inlineStr">
         <is>
-          <t>Software Design as an Aesthetic Design Practice. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E526" t="inlineStr"/>
       <c r="F526" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G526" t="inlineStr"/>
@@ -19767,28 +19767,28 @@
     <row r="527">
       <c r="A527" t="inlineStr">
         <is>
-          <t>01/01/2025</t>
+          <t>01/01/2003</t>
         </is>
       </c>
       <c r="B527" t="inlineStr">
         <is>
-          <t>02/25/2026</t>
+          <t>12/31/2003</t>
         </is>
       </c>
       <c r="C527" t="inlineStr">
         <is>
-          <t>Melemaikalani Moniz</t>
+          <t>Katia Minarikova</t>
         </is>
       </c>
       <c r="D527" t="inlineStr">
         <is>
-          <t>Postdoctoral Fellow in Abundant Soils. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E527" t="inlineStr"/>
       <c r="F527" t="inlineStr">
         <is>
-          <t>Postdoc</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G527" t="inlineStr"/>
@@ -19803,28 +19803,28 @@
     <row r="528">
       <c r="A528" t="inlineStr">
         <is>
-          <t>01/01/2024</t>
+          <t>01/01/2003</t>
         </is>
       </c>
       <c r="B528" t="inlineStr">
         <is>
-          <t>12/31/2026</t>
+          <t>12/31/2003</t>
         </is>
       </c>
       <c r="C528" t="inlineStr">
         <is>
-          <t>Ceyda Yolgörmez</t>
+          <t>Jonathan Joseph</t>
         </is>
       </c>
       <c r="D528" t="inlineStr">
         <is>
-          <t>Horizon Postdoctoral Fellow in Abundant Intelligences. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E528" t="inlineStr"/>
       <c r="F528" t="inlineStr">
         <is>
-          <t>Postdoc</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G528" t="inlineStr"/>
@@ -19839,28 +19839,28 @@
     <row r="529">
       <c r="A529" t="inlineStr">
         <is>
-          <t>01/01/2019</t>
+          <t>01/01/2003</t>
         </is>
       </c>
       <c r="B529" t="inlineStr">
         <is>
-          <t>12/31/2021</t>
+          <t>12/31/2003</t>
         </is>
       </c>
       <c r="C529" t="inlineStr">
         <is>
-          <t>Leuli Eschraghi</t>
+          <t>David Johnston</t>
         </is>
       </c>
       <c r="D529" t="inlineStr">
         <is>
-          <t>Horizon Postdoctoral Fellow in Indigenous Futures. Concordia University.</t>
+          <t>Undergraduate Research Assistant. Concordia University.</t>
         </is>
       </c>
       <c r="E529" t="inlineStr"/>
       <c r="F529" t="inlineStr">
         <is>
-          <t>Postdoc</t>
+          <t>Undergraduate</t>
         </is>
       </c>
       <c r="G529" t="inlineStr"/>

</xml_diff>